<commit_message>
Proyección según tela comprada: Negro 2500 m + Verde 950 m
- Pool compartido Chaqueta Lite + Lite Pant (sin Vinotinto)
- Verde al máximo de metros asignados por modelo
- Negro: rango mín con margen +30% (÷1,30) y máx uso total de tela
- Reparto de tela 48,7% pant / 51,3% chaqueta (peso 1.280 vs 1.350)
- Excel y resumen actualizados

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -645,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.25</v>
+        <v>1.4</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>439.6</v>
+        <v>492.3</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>503.7</v>
+        <v>556.4</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>── COBERTURA Y STOCK DE SEGURIDAD ──</t>
+          <t>── COBERTURA Y STOCK ──</t>
         </is>
       </c>
     </row>
@@ -838,182 +838,191 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Stock de seguridad</t>
+          <t>Stock de seguridad producción</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>+15%</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>sobre demanda teórica</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Demanda teórica mín (sin cap cierres)</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1448</v>
+          <t>Stock de seguridad tela (compra)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>+20%</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>und</t>
+          <t>sobre consumo VIORI</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Demanda teórica máx (sin cap cierres)</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2027</v>
+          <t>Stock PT en taller</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Contemplado</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>buffer operativo pre-distribución y reposición</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Demanda teórica mín (referencia)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>und</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Demanda teórica máx (referencia)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2240</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>── INSUMO LIMITANTE: CIERRES QX NEGRO 0580 ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Inventario global (60 + 75 cm)</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1492</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>und disponibles</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · Cierres 60 cm en stock</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>748</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>und</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · Cierres 75 cm en stock</t>
+          <t>Inventario global (60 + 75 cm)</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>744</v>
+        <v>1492</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>und (adaptables a 60 cm)</t>
+          <t>und disponibles</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Lógica</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>1 cierre = 1 chaqueta · pool global intercambiable</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t xml:space="preserve">  · Cierres 60 cm en stock</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>748</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tope producción (inventario global)</t>
+          <t xml:space="preserve">  · Cierres 75 cm en stock</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1492</v>
+        <v>744</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>und</t>
+          <t>und (adaptables a 60 cm)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>¿Rango 890–970 cabe en stock?</t>
+          <t>Lógica</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>1 cierre = 1 chaqueta · pool global intercambiable</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Tope producción (inventario global)</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1492</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>¿Rango 1280–1350 cabe en stock?</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>SÍ</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>── RANGO DE PRODUCCIÓN (ACORDADO) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>MÍNIMO (compromiso)</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>890</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>MÁXIMO</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>970</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>und</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Rango de acción</t>
+          <t>MÍNIMO (compromiso)</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>80</v>
+        <v>1280</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1024,107 +1033,111 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cierres usados al mínimo</t>
+          <t>MÁXIMO</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>890</v>
+        <v>1350</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>de 1492 disp.</t>
+          <t>und</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cierres usados al máximo</t>
+          <t>Rango de acción</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>970</v>
+        <v>70</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>de 1492 disp.</t>
+          <t>und</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Cierres usados al mínimo</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1280</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>de 1492 disp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Cierres usados al máximo</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1350</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>de 1492 disp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>Remanente global al máximo</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>522</v>
-      </c>
-      <c r="C37" t="inlineStr">
+      <c r="B39" t="n">
+        <v>142</v>
+      </c>
+      <c r="C39" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>── COLORES DE PRODUCCIÓN ──</t>
         </is>
       </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Negro</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>protagonista</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Vinotinto</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Verde Militar</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>protagonista</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Curva completa color × talla</t>
+          <t>Vinotinto</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Hoja Cantidades por Colores</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1132,12 +1145,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Detalle color/talla Mín-Máx</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Hoja Producción Color × Talla</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1145,121 +1158,94 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>Curva completa color × talla</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Hoja Cantidades por Colores</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Detalle color/talla Mín-Máx</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Hoja Producción Color × Talla</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>Compra tela VIORI</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>Hoja Compra de Tela (+20% SS)</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Tolón histórico</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+      <c r="C47" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Tolón proyectado (85% Chacao)</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>und/mes</t>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>── AJUSTE CURVA TALLAS ──</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Web histórica</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>Curva histórica (Jacket 1.0 + 2.0)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Dashboards combinados</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Web proyectada (60% Cerro Verde)</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>37.2</v>
+          <t>XL (+1.5 pp ← L)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>XL 5.1%</t>
+        </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>und/mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>La Vela histórica</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>10</v>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>und/mes</t>
+          <t>hist XL 3.6% · L 13.8% · XS sin cambio</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>77.7</v>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>und/mes</t>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Grand Plaz histórica</t>
+          <t>Tolón histórico</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>8.300000000000001</v>
+        <v>8.1</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1270,11 +1256,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+68% hist.)</t>
+          <t>Tolón proyectado (85% Chacao)</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>14</v>
+        <v>60.4</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1285,11 +1271,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+          <t>Web histórica</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>64.09999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1300,45 +1286,135 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Corporativo</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>EXCLUIDO</t>
+          <t>Web proyectada (60% Cerro Verde)</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>La Vela histórica</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>10</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+          <t>Grand Plaz histórica</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+          <t>Grand Plaz proyectada (+68% hist.)</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>14</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
+        <is>
+          <t>Corporativo</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>EXCLUIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
         <is>
           <t>• Preferencia: 60 cm → XS/S/M · 75 cm → L/XL · excedente 75 cm adaptable a 60 cm.</t>
         </is>
@@ -1377,7 +1453,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>DAMA · Curva Jacket 1.0 + 2.0 DAMA combinado</t>
+          <t>DAMA · Curva Jacket 1.0 + 2.0 DAMA · XL +1.5 pp desde L</t>
         </is>
       </c>
     </row>
@@ -1433,16 +1509,16 @@
         <v>60</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>216</v>
+        <v>310</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>235</v>
+        <v>327</v>
       </c>
       <c r="F5" t="n">
-        <v>216</v>
+        <v>310</v>
       </c>
       <c r="G5" t="n">
-        <v>235</v>
+        <v>327</v>
       </c>
     </row>
     <row r="6">
@@ -1460,16 +1536,16 @@
         <v>60</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>259</v>
+        <v>373</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>283</v>
+        <v>394</v>
       </c>
       <c r="F6" t="n">
-        <v>259</v>
+        <v>373</v>
       </c>
       <c r="G6" t="n">
-        <v>283</v>
+        <v>394</v>
       </c>
     </row>
     <row r="7">
@@ -1487,16 +1563,16 @@
         <v>60</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>247</v>
+        <v>355</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>269</v>
+        <v>374</v>
       </c>
       <c r="F7" t="n">
-        <v>247</v>
+        <v>355</v>
       </c>
       <c r="G7" t="n">
-        <v>269</v>
+        <v>374</v>
       </c>
     </row>
     <row r="8">
@@ -1507,23 +1583,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>13.8%</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>75</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>136</v>
+        <v>176</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>148</v>
+        <v>186</v>
       </c>
       <c r="F8" t="n">
-        <v>136</v>
+        <v>176</v>
       </c>
       <c r="G8" t="n">
-        <v>148</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9">
@@ -1534,23 +1610,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>3.6%</t>
+          <t>5.1%</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>75</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="F9" t="n">
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="G9" t="n">
-        <v>35</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10">
@@ -1560,16 +1636,16 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>722</v>
+        <v>1038</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>787</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="12">
@@ -1583,7 +1659,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Usa máx 970 (65%)</t>
+          <t>Usa máx 1350 (90%)</t>
         </is>
       </c>
     </row>
@@ -1594,11 +1670,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>522</v>
+        <v>142</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Incl. 39 cierres 75→60 cm</t>
+          <t>Incl. 347 cierres 75→60 cm</t>
         </is>
       </c>
     </row>
@@ -1643,14 +1719,14 @@
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Rango producción: 890 – 970 und</t>
+          <t>Rango producción: 1280 – 1350 und</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>MÍNIMO — 890 und (compromiso)</t>
+          <t>MÍNIMO — 1280 und (compromiso)</t>
         </is>
       </c>
     </row>
@@ -1698,22 +1774,22 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>104</v>
+        <v>149</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>99</v>
+        <v>142</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="G7" s="18" t="n">
-        <v>356</v>
+        <v>512</v>
       </c>
     </row>
     <row r="8">
@@ -1723,22 +1799,22 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>74</v>
+        <v>106</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="G8" s="18" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
     </row>
     <row r="9">
@@ -1748,22 +1824,22 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="C9" s="18" t="n">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="D9" s="18" t="n">
-        <v>74</v>
+        <v>106</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="G9" s="18" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
     </row>
     <row r="10">
@@ -1773,28 +1849,28 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>216</v>
+        <v>310</v>
       </c>
       <c r="C10" s="20" t="n">
-        <v>260</v>
+        <v>373</v>
       </c>
       <c r="D10" s="20" t="n">
-        <v>247</v>
+        <v>354</v>
       </c>
       <c r="E10" s="20" t="n">
-        <v>136</v>
+        <v>177</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="G10" s="20" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>MÁXIMO — 970 und (techo)</t>
+          <t>MÁXIMO — 1350 und (techo)</t>
         </is>
       </c>
     </row>
@@ -1842,22 +1918,22 @@
         </is>
       </c>
       <c r="B14" s="18" t="n">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="C14" s="18" t="n">
-        <v>113</v>
+        <v>157</v>
       </c>
       <c r="D14" s="18" t="n">
-        <v>108</v>
+        <v>150</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>388</v>
+        <v>540</v>
       </c>
     </row>
     <row r="15">
@@ -1867,22 +1943,22 @@
         </is>
       </c>
       <c r="B15" s="18" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="C15" s="18" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="D15" s="18" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
     <row r="16">
@@ -1892,22 +1968,22 @@
         </is>
       </c>
       <c r="B16" s="18" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="C16" s="18" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="D16" s="18" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="F16" s="18" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
     <row r="17">
@@ -1917,22 +1993,22 @@
         </is>
       </c>
       <c r="B17" s="20" t="n">
-        <v>236</v>
+        <v>327</v>
       </c>
       <c r="C17" s="20" t="n">
-        <v>283</v>
+        <v>393</v>
       </c>
       <c r="D17" s="20" t="n">
-        <v>270</v>
+        <v>374</v>
       </c>
       <c r="E17" s="20" t="n">
-        <v>147</v>
+        <v>186</v>
       </c>
       <c r="F17" s="20" t="n">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="G17" s="20" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="19">
@@ -1976,10 +2052,10 @@
         </is>
       </c>
       <c r="B21" s="23" t="n">
-        <v>445.85</v>
+        <v>641.34</v>
       </c>
       <c r="C21" s="24" t="n">
-        <v>485.92</v>
+        <v>676.39</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1999,10 +2075,10 @@
         </is>
       </c>
       <c r="B22" s="23" t="n">
-        <v>535.02</v>
+        <v>769.61</v>
       </c>
       <c r="C22" s="24" t="n">
-        <v>583.1</v>
+        <v>811.67</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2011,7 +2087,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>62.718 kg al máx</t>
+          <t>87.301 kg al máx</t>
         </is>
       </c>
     </row>
@@ -2022,10 +2098,10 @@
         </is>
       </c>
       <c r="B23" s="23" t="n">
-        <v>401.18</v>
+        <v>577.21</v>
       </c>
       <c r="C23" s="24" t="n">
-        <v>437.2</v>
+        <v>608.8</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2034,7 +2110,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>47.024 kg al máx</t>
+          <t>65.48 kg al máx</t>
         </is>
       </c>
     </row>
@@ -2045,10 +2121,10 @@
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>401.18</v>
+        <v>577.21</v>
       </c>
       <c r="C24" s="24" t="n">
-        <v>437.2</v>
+        <v>608.8</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2057,7 +2133,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>47.024 kg al máx</t>
+          <t>65.48 kg al máx</t>
         </is>
       </c>
     </row>
@@ -2068,10 +2144,10 @@
         </is>
       </c>
       <c r="B25" s="23" t="n">
-        <v>1337.39</v>
+        <v>1924.03</v>
       </c>
       <c r="C25" s="24" t="n">
-        <v>1457.5</v>
+        <v>2029.26</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2080,7 +2156,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>156.767 kg al máx · SS 20%</t>
+          <t>218.262 kg al máx · SS 20%</t>
         </is>
       </c>
     </row>
@@ -2091,10 +2167,10 @@
         </is>
       </c>
       <c r="B26" s="23" t="n">
-        <v>440.09</v>
+        <v>633.15</v>
       </c>
       <c r="C26" s="24" t="n">
-        <v>479.65</v>
+        <v>667.76</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2114,10 +2190,10 @@
         </is>
       </c>
       <c r="B27" s="23" t="n">
-        <v>475.69</v>
+        <v>684.35</v>
       </c>
       <c r="C27" s="24" t="n">
-        <v>518.45</v>
+        <v>721.76</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2137,10 +2213,10 @@
         </is>
       </c>
       <c r="B28" s="23" t="n">
-        <v>173.09</v>
+        <v>249.15</v>
       </c>
       <c r="C28" s="24" t="n">
-        <v>188.65</v>
+        <v>262.76</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2160,10 +2236,10 @@
         </is>
       </c>
       <c r="B29" s="23" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
       <c r="C29" s="24" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2172,7 +2248,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pool global 1492 und · rem. 522 al máx</t>
+          <t>Pool global 1492 und · rem. 142 al máx</t>
         </is>
       </c>
     </row>
@@ -2183,10 +2259,10 @@
         </is>
       </c>
       <c r="B30" s="26" t="n">
-        <v>722</v>
+        <v>1038</v>
       </c>
       <c r="C30" s="26" t="n">
-        <v>787</v>
+        <v>1095</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2206,10 +2282,10 @@
         </is>
       </c>
       <c r="B31" s="26" t="n">
-        <v>168</v>
+        <v>242</v>
       </c>
       <c r="C31" s="26" t="n">
-        <v>183</v>
+        <v>255</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2273,7 +2349,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Rango global: 890 – 970 und</t>
+          <t>Rango global: 1280 – 1350 und</t>
         </is>
       </c>
     </row>
@@ -2375,34 +2451,34 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>104</v>
+        <v>149</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>113</v>
+        <v>157</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>99</v>
+        <v>142</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>108</v>
+        <v>150</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -2412,10 +2488,10 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>356</v>
+        <v>512</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>388</v>
+        <v>540</v>
       </c>
     </row>
     <row r="11">
@@ -2516,34 +2592,34 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>74</v>
+        <v>106</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -2553,10 +2629,10 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
     <row r="17">
@@ -2657,34 +2733,34 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>74</v>
+        <v>106</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21">
@@ -2694,10 +2770,10 @@
         </is>
       </c>
       <c r="B21" s="10" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="C21" s="10" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
     <row r="23">
@@ -2707,10 +2783,10 @@
         </is>
       </c>
       <c r="B23" s="10" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="25">
@@ -2727,10 +2803,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>356</v>
+        <v>512</v>
       </c>
       <c r="C26" t="n">
-        <v>388</v>
+        <v>540</v>
       </c>
     </row>
     <row r="27">
@@ -2740,10 +2816,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="C27" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
     <row r="28">
@@ -2753,10 +2829,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="C28" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>
@@ -2883,28 +2959,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>356</v>
+        <v>512</v>
       </c>
       <c r="D5" t="n">
-        <v>388</v>
+        <v>540</v>
       </c>
       <c r="E5" t="n">
-        <v>445.85</v>
+        <v>641.34</v>
       </c>
       <c r="F5" t="n">
-        <v>485.92</v>
+        <v>676.39</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>535.02</v>
+        <v>769.61</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>583.1</v>
+        <v>811.67</v>
       </c>
       <c r="I5" s="23" t="n">
-        <v>57.546</v>
+        <v>82.777</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>62.718</v>
+        <v>87.301</v>
       </c>
     </row>
     <row r="6">
@@ -2919,28 +2995,28 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="D6" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
       <c r="E6" t="n">
-        <v>334.32</v>
+        <v>481.01</v>
       </c>
       <c r="F6" t="n">
-        <v>364.33</v>
+        <v>507.33</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>401.18</v>
+        <v>577.21</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>437.2</v>
+        <v>608.8</v>
       </c>
       <c r="I6" s="23" t="n">
-        <v>43.151</v>
+        <v>62.083</v>
       </c>
       <c r="J6" s="24" t="n">
-        <v>47.024</v>
+        <v>65.48</v>
       </c>
     </row>
     <row r="7">
@@ -2955,28 +3031,28 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="D7" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
       <c r="E7" t="n">
-        <v>334.32</v>
+        <v>481.01</v>
       </c>
       <c r="F7" t="n">
-        <v>364.33</v>
+        <v>507.33</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>401.18</v>
+        <v>577.21</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>437.2</v>
+        <v>608.8</v>
       </c>
       <c r="I7" s="23" t="n">
-        <v>43.151</v>
+        <v>62.083</v>
       </c>
       <c r="J7" s="24" t="n">
-        <v>47.024</v>
+        <v>65.48</v>
       </c>
     </row>
     <row r="8">
@@ -2986,28 +3062,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
       <c r="D8" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
       <c r="E8" t="n">
-        <v>1114.49</v>
+        <v>1603.36</v>
       </c>
       <c r="F8" t="n">
-        <v>1214.58</v>
+        <v>1691.05</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>1337.39</v>
+        <v>1924.03</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>1457.5</v>
+        <v>2029.26</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>143.848</v>
+        <v>206.944</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>156.767</v>
+        <v>218.262</v>
       </c>
     </row>
     <row r="10">
@@ -3076,31 +3152,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="C12" t="n">
-        <v>113</v>
+        <v>157</v>
       </c>
       <c r="D12" t="n">
-        <v>108</v>
+        <v>150</v>
       </c>
       <c r="E12" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="F12" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="G12" t="n">
-        <v>388</v>
+        <v>540</v>
       </c>
       <c r="H12" t="n">
-        <v>485.92</v>
+        <v>676.39</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>583.1</v>
+        <v>811.67</v>
       </c>
       <c r="J12" t="n">
-        <v>62.718</v>
+        <v>87.301</v>
       </c>
     </row>
     <row r="13">
@@ -3110,31 +3186,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="C13" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="D13" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="E13" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="F13" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="G13" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
       <c r="H13" t="n">
-        <v>364.33</v>
+        <v>507.33</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>437.2</v>
+        <v>608.8</v>
       </c>
       <c r="J13" t="n">
-        <v>47.024</v>
+        <v>65.48</v>
       </c>
     </row>
     <row r="14">
@@ -3144,31 +3220,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="C14" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="D14" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="E14" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="F14" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="G14" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
       <c r="H14" t="n">
-        <v>364.33</v>
+        <v>507.33</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>437.2</v>
+        <v>608.8</v>
       </c>
       <c r="J14" t="n">
-        <v>47.024</v>
+        <v>65.48</v>
       </c>
     </row>
     <row r="16">
@@ -3268,10 +3344,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>440.09</v>
+        <v>633.15</v>
       </c>
       <c r="C22" t="n">
-        <v>479.65</v>
+        <v>667.76</v>
       </c>
     </row>
     <row r="23">
@@ -3281,10 +3357,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>475.69</v>
+        <v>684.35</v>
       </c>
       <c r="C23" t="n">
-        <v>518.45</v>
+        <v>721.76</v>
       </c>
     </row>
     <row r="24">
@@ -3294,10 +3370,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>173.09</v>
+        <v>249.15</v>
       </c>
       <c r="C24" t="n">
-        <v>188.65</v>
+        <v>262.76</v>
       </c>
     </row>
   </sheetData>
@@ -3435,34 +3511,34 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="C5" s="24" t="n">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="D5" s="23" t="n">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="E5" s="24" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="H5" s="23" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="J5" s="23" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K5" s="24" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -3472,34 +3548,34 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="D6" s="23" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I6" s="24" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K6" s="24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -3509,34 +3585,34 @@
         </is>
       </c>
       <c r="B7" s="23" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="C7" s="24" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="D7" s="23" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="E7" s="24" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F7" s="23" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="H7" s="23" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I7" s="24" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K7" s="24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -3546,34 +3622,34 @@
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C8" s="24" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="F8" s="23" t="n">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="J8" s="23" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K8" s="24" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -3583,34 +3659,34 @@
         </is>
       </c>
       <c r="B9" s="23" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D9" s="23" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E9" s="24" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F9" s="23" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H9" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I9" s="24" t="n">
-        <v>4</v>
-      </c>
-      <c r="J9" s="26" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="J9" s="23" t="n">
+        <v>1</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -3620,34 +3696,34 @@
         </is>
       </c>
       <c r="B10" s="23" t="n">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="C10" s="24" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D10" s="23" t="n">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E10" s="24" t="n">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="F10" s="23" t="n">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="I10" s="24" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J10" s="23" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="K10" s="24" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -3657,34 +3733,34 @@
         </is>
       </c>
       <c r="B11" s="23" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="C11" s="24" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="E11" s="24" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="F11" s="23" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="H11" s="23" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I11" s="24" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="J11" s="23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -3694,34 +3770,34 @@
         </is>
       </c>
       <c r="B12" s="23" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C12" s="24" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E12" s="24" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F12" s="23" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="G12" s="24" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H12" s="23" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I12" s="24" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J12" s="23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K12" s="24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -3731,34 +3807,34 @@
         </is>
       </c>
       <c r="B13" s="23" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="C13" s="24" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D13" s="23" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="E13" s="24" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="F13" s="23" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G13" s="24" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="H13" s="23" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="I13" s="24" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="J13" s="23" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -3768,34 +3844,34 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>216</v>
+        <v>312</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>235</v>
+        <v>329</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>260</v>
+        <v>374</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>283</v>
+        <v>394</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>245</v>
+        <v>355</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>270</v>
+        <v>375</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>137</v>
+        <v>176</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>149</v>
+        <v>186</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>33</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16">
@@ -3834,10 +3910,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>154</v>
+        <v>221</v>
       </c>
       <c r="C18" t="n">
-        <v>169</v>
+        <v>233</v>
       </c>
       <c r="D18" t="n">
         <v>93.3</v>
@@ -3850,10 +3926,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>100</v>
+        <v>144</v>
       </c>
       <c r="C19" t="n">
-        <v>109</v>
+        <v>152</v>
       </c>
       <c r="D19" t="n">
         <v>61</v>
@@ -3866,10 +3942,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>102</v>
+        <v>147</v>
       </c>
       <c r="C20" t="n">
-        <v>111</v>
+        <v>155</v>
       </c>
       <c r="D20" t="n">
         <v>62.1</v>
@@ -3882,10 +3958,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>117</v>
+        <v>168</v>
       </c>
       <c r="C21" t="n">
-        <v>127</v>
+        <v>177</v>
       </c>
       <c r="D21" t="n">
         <v>71</v>
@@ -3898,10 +3974,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="C22" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D22" t="n">
         <v>14</v>
@@ -3914,10 +3990,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>128</v>
+        <v>184</v>
       </c>
       <c r="C23" t="n">
-        <v>139</v>
+        <v>194</v>
       </c>
       <c r="D23" t="n">
         <v>77.7</v>
@@ -3930,10 +4006,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>99</v>
+        <v>143</v>
       </c>
       <c r="C24" t="n">
-        <v>108</v>
+        <v>151</v>
       </c>
       <c r="D24" t="n">
         <v>60.4</v>
@@ -3946,10 +4022,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>61</v>
+        <v>88</v>
       </c>
       <c r="C25" t="n">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="D25" t="n">
         <v>37.2</v>
@@ -3962,10 +4038,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>106</v>
+        <v>152</v>
       </c>
       <c r="C26" t="n">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="D26" t="n">
         <v>64.09999999999999</v>
@@ -4149,10 +4225,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>722</v>
+        <v>1038</v>
       </c>
       <c r="D14" t="n">
-        <v>787</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="15">
@@ -4167,10 +4243,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>168</v>
+        <v>242</v>
       </c>
       <c r="D15" t="n">
-        <v>183</v>
+        <v>255</v>
       </c>
     </row>
     <row r="16">
@@ -4181,16 +4257,16 @@
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
       <c r="D16" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>── ASIGNACIÓN AL MÁXIMO (970 und) ──</t>
+          <t>── ASIGNACIÓN AL MÁXIMO (1350 und) ──</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4299,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>39</v>
+        <v>347</v>
       </c>
     </row>
     <row r="22">
@@ -4233,7 +4309,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>183</v>
+        <v>255</v>
       </c>
     </row>
     <row r="23">
@@ -4243,7 +4319,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>222</v>
+        <v>602</v>
       </c>
     </row>
     <row r="24">
@@ -4253,7 +4329,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="25">
@@ -4263,7 +4339,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>522</v>
+        <v>142</v>
       </c>
     </row>
     <row r="27">
@@ -4274,7 +4350,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>890 – 970 und</t>
+          <t>1280 – 1350 und</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A46"/>
+  <dimension ref="A1:A56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -4358,149 +4434,149 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Factor ×1.25 (diciembre). Diciembre 2025 combinado: 685 und.</t>
+          <t xml:space="preserve">   Factor ×1.4 (diciembre — incrementado para escenario temporada alta).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Diciembre 2025 combinado: 685 und.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>3. AJUSTES DE TIENDA (según indicación)</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Tolón: proyectado al 85% de Chacao (71 → 60 und/mes).</t>
+          <t xml:space="preserve">   STOCK DE SEGURIDAD Y TALLER</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Histórico Tolón: 8 und/mes — subestimado por tienda nueva.</t>
+          <t xml:space="preserve">   • Producción: +15% SS sobre demanda teórica.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Web: proyectada al 60% de Cerro Verde (62 → 37 und/mes).</t>
+          <t xml:space="preserve">   • Tela (compra): +20% SS sobre consumo VIORI.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Histórico Web: 8 und/mes.</t>
+          <t xml:space="preserve">   • Producto terminado en taller: buffer operativo (pre-distribución a tiendas y reposición).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • La Vela (nueva): promedio Sambil + Cerro Verde = 78 und/mes.</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     Histórico La Vela: 10 und/mes.</t>
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>3. AJUSTES DE TIENDA (según indicación)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Grand Plaz: histórico × 1.68 (+68%) = 14 und/mes.</t>
+          <t xml:space="preserve">   • Tolón: proyectado al 85% de Chacao (71 → 60 und/mes).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Histórico Grand Plaz: 8 und/mes.</t>
+          <t xml:space="preserve">     Histórico Tolón: 8 und/mes — subestimado por tienda nueva.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Barquisimeto (nueva): promedio Grieta + Chacao + Tolón proyectado = 64 und/mes.</t>
+          <t xml:space="preserve">   • Web: proyectada al 60% de Cerro Verde (62 → 37 und/mes).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Corporativo: EXCLUIDO.</t>
+          <t xml:space="preserve">     Histórico Web: 8 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • La Vela (nueva): promedio Sambil + Cerro Verde = 78 und/mes.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>4. RANGO GLOBAL ACORDADO</t>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Histórico La Vela: 10 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Mínimo: 890 und | Máximo: 970 und.</t>
+          <t xml:space="preserve">   • Grand Plaz: histórico × 1.68 (+68%) = 14 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Demanda teórica calculada: 1448 – 2027 und (referencia).</t>
+          <t xml:space="preserve">     Histórico Grand Plaz: 8 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Barquisimeto (nueva): promedio Grieta + Chacao + Tolón proyectado = 64 und/mes.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
-        <is>
-          <t>5. INSUMO LIMITANTE — CIERRES (INVENTARIO GLOBAL)</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Corporativo: EXCLUIDO.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Stock total: 748 (60 cm) + 744 (75 cm) = 1492 und.</t>
-        </is>
-      </c>
+      <c r="A28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Los cierres 75 cm se adaptan a 60 cm → se considera pool global intercambiable.</t>
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>4. RANGO GLOBAL ACORDADO</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Tope producción = 1492 und (1 cierre por chaqueta).</t>
+          <t xml:space="preserve">   Mínimo: 1280 und | Máximo: 1350 und.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Al máximo (970 und) quedan 522 cierres remanentes.</t>
+          <t xml:space="preserve">   Demanda teórica calculada: 1600 – 2240 und (referencia).</t>
         </is>
       </c>
     </row>
@@ -4510,88 +4586,150 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>6. RANGO MÍNIMO / MÁXIMO</t>
+          <t>5. INSUMO LIMITANTE — CIERRES (INVENTARIO GLOBAL)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Compromiso mín: 890 und.</t>
+          <t xml:space="preserve">   Stock total: 748 (60 cm) + 744 (75 cm) = 1492 und.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Techo máx: 970 und.</t>
+          <t xml:space="preserve">   Los cierres 75 cm se adaptan a 60 cm → se considera pool global intercambiable.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Tope producción = 1492 und (1 cierre por chaqueta).</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
-        <is>
-          <t>7. DISTRIBUCIÓN</t>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Al máximo (1350 und) quedan 142 cierres remanentes.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
-        </is>
-      </c>
+      <c r="A38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Por talla: curva combinada Jacket 1.0 + 2.0 DAMA.</t>
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>6. RANGO MÍNIMO / MÁXIMO</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Compromiso mín: 1280 und.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="inlineStr">
-        <is>
-          <t>8. COLORES Y COMPRA DE TELA</t>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Techo máx: 1350 und.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Colores: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
-        </is>
-      </c>
+      <c r="A42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>7. AJUSTE CURVA TALLAS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Consumo VIORI por pieza (ficha técnica): XS 1.19m · S 1.22m · M 1.28m · L 1.34m · XL 1.35m.</t>
+          <t xml:space="preserve">   Histórica Jacket 1.0 + 2.0 DAMA: L 15.3% · XL 3.6%.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t xml:space="preserve">   XL reforzado +1.5 pp desde L → L 13.8% · XL 5.1% (XS sin cambio).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>8. DISTRIBUCIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Por talla: curva histórica ajustada (ver sección 7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>9. COLORES Y COMPRA DE TELA</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Colores: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Consumo VIORI por pieza (ficha técnica): XS 1.19m · S 1.22m · M 1.28m · L 1.34m · XL 1.35m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Stock de seguridad tela: +20% sobre consumo (compra = consumo × 1.2).</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t xml:space="preserve">   Ver hojas 'Producción Color × Talla' y 'Compra de Tela VIORI'.</t>
         </is>

</xml_diff>

<commit_message>
Min/máx por color: verde y negro con rangos distintos en Excel
- Verde: mín ÷1,30 · máx 100% tela asignada
- Negro: mín ÷1,15 (mín más alto) · máx 100% tela
- Bloques MÍNIMO y MÁXIMO ya no repiten las mismas und en verde

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -88,7 +88,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -152,11 +152,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="008B2942"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="004B5320"/>
       </patternFill>
     </fill>
@@ -192,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -271,11 +266,8 @@
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -645,7 +637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -999,7 +991,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>¿Rango 1280–1350 cabe en stock?</t>
+          <t>¿Producción cabe en cierres?</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1011,7 +1003,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>── RANGO DE PRODUCCIÓN (ACORDADO) ──</t>
+          <t>── RANGO DE PRODUCCIÓN ──</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1014,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1280</v>
+        <v>1189</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1037,7 +1029,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1350</v>
+        <v>1413</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1052,7 +1044,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>70</v>
+        <v>224</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1067,7 +1059,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1280</v>
+        <v>1189</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1082,7 +1074,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1350</v>
+        <v>1413</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1097,7 +1089,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>142</v>
+        <v>79</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1108,313 +1100,446 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>── COLORES DE PRODUCCIÓN ──</t>
+          <t>── TELA DISPONIBLE (POOL CHAQUETA + PANT) ──</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Negro</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
+          <t>Negro comprado (total)</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2500</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>protagonista</t>
+          <t>mts</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Vinotinto</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
+          <t>Verde Militar comprado (total)</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>950</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>mts</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Verde Militar</t>
+          <t>Reparto tela este modelo</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
+          <t>51.3%</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>peso 1.280 vs 1.350</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Curva completa color × talla</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Hoja Cantidades por Colores</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr"/>
+          <t>Verde — unidades mín (÷1.3)</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>299</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Detalle color/talla Mín-Máx</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Hoja Producción Color × Talla</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr"/>
+          <t>Verde — unidades máx (100% tela)</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>389</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Compra tela VIORI</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Hoja Compra de Tela (+20% SS)</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr"/>
+          <t>Negro — unidades mín (÷1.15)</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>890</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Negro — unidades máx (100% tela)</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1024</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>── AJUSTE CURVA TALLAS ──</t>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Consumo prom. VIORI/pieza (curva tallas)</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1.2525</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>mts</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Curva histórica (Jacket 1.0 + 2.0)</t>
+          <t>Vinotinto</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Dashboards combinados</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>XL (+1.5 pp ← L)</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>XL 5.1%</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>hist XL 3.6% · L 13.8% · XS sin cambio</t>
+          <t>NO COMPRADO</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>── COLORES DE PRODUCCIÓN ──</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>890</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>mín · máx 1024 und</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Tolón histórico</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>8.1</v>
+        <v>299</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>und/mes</t>
+          <t>mín · máx 389 und</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Tolón proyectado (85% Chacao)</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>Curva completa color × talla</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Hoja Cantidades por Colores</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Web histórica</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>Detalle color/talla Mín-Máx</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Hoja Producción Color × Talla</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Web proyectada (60% Cerro Verde)</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>37.2</v>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>La Vela histórica</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>10</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>Compra tela VIORI</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Hoja Compra de Tela (+20% SS)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>77.7</v>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>und/mes</t>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>── AJUSTE CURVA TALLAS ──</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Grand Plaz histórica</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>Curva histórica (Jacket 1.0 + 2.0)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Dashboards combinados</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+68% hist.)</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>14</v>
+          <t>XL (+1.5 pp ← L)</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>XL 5.1%</t>
+        </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
+          <t>hist XL 3.6% · L 13.8% · XS sin cambio</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Tolón histórico</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
           <t>und/mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>64.09999999999999</v>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Corporativo</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>EXCLUIDO</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>Tolón proyectado (85% Chacao)</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+          <t>Web histórica</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+          <t>Web proyectada (60% Cerro Verde)</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>La Vela histórica</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>10</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
+        <is>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Grand Plaz histórica</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Grand Plaz proyectada (+68% hist.)</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>14</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Corporativo</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>EXCLUIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
         <is>
           <t>• Preferencia: 60 cm → XS/S/M · 75 cm → L/XL · excedente 75 cm adaptable a 60 cm.</t>
         </is>
@@ -1509,16 +1634,16 @@
         <v>60</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>310</v>
+        <v>288</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>327</v>
+        <v>343</v>
       </c>
       <c r="F5" t="n">
-        <v>310</v>
+        <v>288</v>
       </c>
       <c r="G5" t="n">
-        <v>327</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6">
@@ -1536,16 +1661,16 @@
         <v>60</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>373</v>
+        <v>347</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>394</v>
+        <v>412</v>
       </c>
       <c r="F6" t="n">
-        <v>373</v>
+        <v>347</v>
       </c>
       <c r="G6" t="n">
-        <v>394</v>
+        <v>412</v>
       </c>
     </row>
     <row r="7">
@@ -1563,16 +1688,16 @@
         <v>60</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>355</v>
+        <v>330</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>374</v>
+        <v>392</v>
       </c>
       <c r="F7" t="n">
-        <v>355</v>
+        <v>330</v>
       </c>
       <c r="G7" t="n">
-        <v>374</v>
+        <v>392</v>
       </c>
     </row>
     <row r="8">
@@ -1590,16 +1715,16 @@
         <v>75</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="F8" t="n">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="G8" t="n">
-        <v>186</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9">
@@ -1617,16 +1742,16 @@
         <v>75</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F9" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="G9" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10">
@@ -1636,16 +1761,16 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>1280</v>
+        <v>1189</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>1350</v>
+        <v>1413</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>1038</v>
+        <v>965</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>1095</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="12">
@@ -1659,7 +1784,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Usa máx 1350 (90%)</t>
+          <t>Usa máx 1413 (95%)</t>
         </is>
       </c>
     </row>
@@ -1670,11 +1795,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>142</v>
+        <v>79</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Incl. 347 cierres 75→60 cm</t>
+          <t>Incl. 399 cierres 75→60 cm</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1712,21 +1837,21 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>CHAQUETA LITE · Proporción Negro 40% · Vinotinto 30% · Verde Militar 30%</t>
+          <t>Tela disponible Negro + Verde Militar (pool compartido con Lite Pant)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Rango producción: 1280 – 1350 und</t>
+          <t>Rango producción: 1189 – 1413 und</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>MÍNIMO — 1280 und (compromiso)</t>
+          <t>MÍNIMO — 1189 und (compromiso)</t>
         </is>
       </c>
     </row>
@@ -1774,288 +1899,284 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>124</v>
+        <v>216</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>149</v>
+        <v>259</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>142</v>
+        <v>247</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>71</v>
+        <v>123</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="G7" s="18" t="n">
-        <v>512</v>
+        <v>890</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>Vinotinto · 30%</t>
+          <t>Verde Militar · 30%</t>
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G8" s="18" t="n">
-        <v>384</v>
+        <v>299</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>Verde Militar · 30%</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="n">
-        <v>93</v>
-      </c>
-      <c r="C9" s="18" t="n">
-        <v>112</v>
-      </c>
-      <c r="D9" s="18" t="n">
-        <v>106</v>
-      </c>
-      <c r="E9" s="18" t="n">
-        <v>53</v>
-      </c>
-      <c r="F9" s="18" t="n">
-        <v>20</v>
-      </c>
-      <c r="G9" s="18" t="n">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B10" s="20" t="n">
-        <v>310</v>
-      </c>
-      <c r="C10" s="20" t="n">
-        <v>373</v>
-      </c>
-      <c r="D10" s="20" t="n">
-        <v>354</v>
-      </c>
-      <c r="E10" s="20" t="n">
-        <v>177</v>
-      </c>
-      <c r="F10" s="20" t="n">
-        <v>66</v>
-      </c>
-      <c r="G10" s="20" t="n">
-        <v>1280</v>
+      <c r="B9" s="20" t="n">
+        <v>289</v>
+      </c>
+      <c r="C9" s="20" t="n">
+        <v>346</v>
+      </c>
+      <c r="D9" s="20" t="n">
+        <v>330</v>
+      </c>
+      <c r="E9" s="20" t="n">
+        <v>164</v>
+      </c>
+      <c r="F9" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>1189</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>MÁXIMO — 1413 und (techo)</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>MÁXIMO — 1350 und (techo)</t>
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>CHAQUETA LITE DAMA</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>Tot</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>CHAQUETA LITE DAMA</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>XS</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E13" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="F13" s="16" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
-      </c>
-      <c r="G13" s="16" t="inlineStr">
-        <is>
-          <t>Tot</t>
-        </is>
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Negro · 40%</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n">
+        <v>248</v>
+      </c>
+      <c r="C13" s="18" t="n">
+        <v>299</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>284</v>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>141</v>
+      </c>
+      <c r="F13" s="18" t="n">
+        <v>52</v>
+      </c>
+      <c r="G13" s="18" t="n">
+        <v>1024</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>Negro · 40%</t>
+          <t>Verde Militar · 30%</t>
         </is>
       </c>
       <c r="B14" s="18" t="n">
-        <v>131</v>
+        <v>94</v>
       </c>
       <c r="C14" s="18" t="n">
-        <v>157</v>
+        <v>113</v>
       </c>
       <c r="D14" s="18" t="n">
-        <v>150</v>
+        <v>108</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>540</v>
+        <v>389</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>Vinotinto · 30%</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="n">
-        <v>98</v>
-      </c>
-      <c r="C15" s="18" t="n">
-        <v>118</v>
-      </c>
-      <c r="D15" s="18" t="n">
-        <v>112</v>
-      </c>
-      <c r="E15" s="18" t="n">
-        <v>56</v>
-      </c>
-      <c r="F15" s="18" t="n">
-        <v>21</v>
-      </c>
-      <c r="G15" s="18" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Verde Militar · 30%</t>
-        </is>
-      </c>
-      <c r="B16" s="18" t="n">
-        <v>98</v>
-      </c>
-      <c r="C16" s="18" t="n">
-        <v>118</v>
-      </c>
-      <c r="D16" s="18" t="n">
-        <v>112</v>
-      </c>
-      <c r="E16" s="18" t="n">
-        <v>56</v>
-      </c>
-      <c r="F16" s="18" t="n">
-        <v>21</v>
-      </c>
-      <c r="G16" s="18" t="n">
-        <v>405</v>
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>342</v>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>412</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <v>392</v>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>195</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <v>72</v>
+      </c>
+      <c r="G15" s="20" t="n">
+        <v>1413</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>TOTAL GENERAL</t>
-        </is>
-      </c>
-      <c r="B17" s="20" t="n">
-        <v>327</v>
-      </c>
-      <c r="C17" s="20" t="n">
-        <v>393</v>
-      </c>
-      <c r="D17" s="20" t="n">
-        <v>374</v>
-      </c>
-      <c r="E17" s="20" t="n">
-        <v>186</v>
-      </c>
-      <c r="F17" s="20" t="n">
-        <v>70</v>
-      </c>
-      <c r="G17" s="20" t="n">
-        <v>1350</v>
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>── INSUMOS PARA COMPRA (Mín / Máx) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Insumo</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
-        <is>
-          <t>── INSUMOS PARA COMPRA (Mín / Máx) ──</t>
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>Tela VIORI — Negro (consumo)</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="n">
+        <v>1114.75</v>
+      </c>
+      <c r="C19" s="24" t="n">
+        <v>1282.56</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>metros</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Tela en bodega</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Insumo</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Mín</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Máx</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Unidad</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Nota</t>
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>Tela VIORI — Verde Militar (consumo)</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="n">
+        <v>374.44</v>
+      </c>
+      <c r="C20" s="24" t="n">
+        <v>487.32</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>metros</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Tela en bodega</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="22" t="inlineStr">
         <is>
-          <t>Tela VIORI — Negro (consumo)</t>
+          <t>TOTAL tela VIORI</t>
         </is>
       </c>
       <c r="B21" s="23" t="n">
-        <v>641.34</v>
+        <v>1489.19</v>
       </c>
       <c r="C21" s="24" t="n">
-        <v>676.39</v>
+        <v>1769.88</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2064,21 +2185,21 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sin SS</t>
+          <t>190.364 kg al máx · consumo = tela disponible</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="22" t="inlineStr">
         <is>
-          <t>Tela VIORI — Negro (compra +SS)</t>
+          <t>Elástica 4.5 cm</t>
         </is>
       </c>
       <c r="B22" s="23" t="n">
-        <v>769.61</v>
+        <v>588.11</v>
       </c>
       <c r="C22" s="24" t="n">
-        <v>811.67</v>
+        <v>698.89</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2087,21 +2208,21 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>87.301 kg al máx</t>
+          <t>Ficha técnica</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="22" t="inlineStr">
         <is>
-          <t>Tela VIORI — Vinotinto (compra +SS)</t>
+          <t>Sesgo cintura 2 cm</t>
         </is>
       </c>
       <c r="B23" s="23" t="n">
-        <v>577.21</v>
+        <v>635.67</v>
       </c>
       <c r="C23" s="24" t="n">
-        <v>608.8</v>
+        <v>755.41</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2110,21 +2231,21 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>65.48 kg al máx</t>
+          <t>Ficha técnica</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="22" t="inlineStr">
         <is>
-          <t>Tela VIORI — Verde Militar (compra +SS)</t>
+          <t>Sesgo manga 2 cm</t>
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>577.21</v>
+        <v>231.41</v>
       </c>
       <c r="C24" s="24" t="n">
-        <v>608.8</v>
+        <v>274.99</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2133,166 +2254,74 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>65.48 kg al máx</t>
+          <t>Ficha técnica</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="22" t="inlineStr">
         <is>
-          <t>TOTAL tela VIORI (compra +SS)</t>
+          <t>Cierres QX Negro 0580</t>
         </is>
       </c>
       <c r="B25" s="23" t="n">
-        <v>1924.03</v>
+        <v>1189</v>
       </c>
       <c r="C25" s="24" t="n">
-        <v>2029.26</v>
+        <v>1413</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>metros</t>
+          <t>und</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>218.262 kg al máx · SS 20%</t>
+          <t>Pool global 1492 und · rem. 79 al máx</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="22" t="inlineStr">
-        <is>
-          <t>Elástica 4.5 cm</t>
-        </is>
-      </c>
-      <c r="B26" s="23" t="n">
-        <v>633.15</v>
-      </c>
-      <c r="C26" s="24" t="n">
-        <v>667.76</v>
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · Preferencia 60 cm (XS/S/M)</t>
+        </is>
+      </c>
+      <c r="B26" s="26" t="n">
+        <v>965</v>
+      </c>
+      <c r="C26" s="26" t="n">
+        <v>1147</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>metros</t>
+          <t>und</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Ficha técnica</t>
+          <t>Stock 748 und</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="inlineStr">
-        <is>
-          <t>Sesgo cintura 2 cm</t>
-        </is>
-      </c>
-      <c r="B27" s="23" t="n">
-        <v>684.35</v>
-      </c>
-      <c r="C27" s="24" t="n">
-        <v>721.76</v>
+      <c r="A27" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · Preferencia 75 cm (L/XL)</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="n">
+        <v>224</v>
+      </c>
+      <c r="C27" s="26" t="n">
+        <v>266</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>metros</t>
+          <t>und</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
-        <is>
-          <t>Ficha técnica</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="22" t="inlineStr">
-        <is>
-          <t>Sesgo manga 2 cm</t>
-        </is>
-      </c>
-      <c r="B28" s="23" t="n">
-        <v>249.15</v>
-      </c>
-      <c r="C28" s="24" t="n">
-        <v>262.76</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>metros</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Ficha técnica</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="22" t="inlineStr">
-        <is>
-          <t>Cierres QX Negro 0580</t>
-        </is>
-      </c>
-      <c r="B29" s="23" t="n">
-        <v>1280</v>
-      </c>
-      <c r="C29" s="24" t="n">
-        <v>1350</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Pool global 1492 und · rem. 142 al máx</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · Preferencia 60 cm (XS/S/M)</t>
-        </is>
-      </c>
-      <c r="B30" s="26" t="n">
-        <v>1038</v>
-      </c>
-      <c r="C30" s="26" t="n">
-        <v>1095</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Stock 748 und</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · Preferencia 75 cm (L/XL)</t>
-        </is>
-      </c>
-      <c r="B31" s="26" t="n">
-        <v>242</v>
-      </c>
-      <c r="C31" s="26" t="n">
-        <v>255</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
         <is>
           <t>Stock 744 und · adaptable</t>
         </is>
@@ -2302,8 +2331,8 @@
   <mergeCells count="5">
     <mergeCell ref="A6"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A13"/>
+    <mergeCell ref="A12"/>
+    <mergeCell ref="A11:G11"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2316,7 +2345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2342,21 +2371,21 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Proporción: Negro 40% · Vinotinto 30% · Verde Militar 30%</t>
+          <t>Colores según tela disponible (Negro + Verde Militar)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Rango global: 1280 – 1350 und</t>
+          <t>Rango global: 1189 – 1413 und</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>Negro (40%)</t>
+          <t>Negro (1024 und máx)</t>
         </is>
       </c>
     </row>
@@ -2451,34 +2480,34 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>124</v>
+        <v>216</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>131</v>
+        <v>248</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>149</v>
+        <v>259</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>157</v>
+        <v>299</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>142</v>
+        <v>247</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>150</v>
+        <v>284</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>71</v>
+        <v>123</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>74</v>
+        <v>141</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9">
@@ -2488,16 +2517,16 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>512</v>
+        <v>890</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>540</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
         <is>
-          <t>Vinotinto (30%)</t>
+          <t>Verde Militar (389 und máx)</t>
         </is>
       </c>
     </row>
@@ -2592,34 +2621,34 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J14" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="K14" s="8" t="n">
         <v>20</v>
-      </c>
-      <c r="K14" s="8" t="n">
-        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -2629,233 +2658,73 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>384</v>
+        <v>299</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>405</v>
+        <v>389</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="30" t="inlineStr">
-        <is>
-          <t>Verde Militar (30%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="28" t="inlineStr">
-        <is>
-          <t>Talla</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>XS</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>1189</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>1413</v>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Mín</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Máx</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Mín</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Máx</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Mín</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>Máx</t>
-        </is>
-      </c>
-      <c r="H19" s="7" t="inlineStr">
-        <is>
-          <t>Mín</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="inlineStr">
-        <is>
-          <t>Máx</t>
-        </is>
-      </c>
-      <c r="J19" s="7" t="inlineStr">
-        <is>
-          <t>Mín</t>
-        </is>
-      </c>
-      <c r="K19" s="8" t="inlineStr">
-        <is>
-          <t>Máx</t>
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Resumen por color (Mín / Máx):</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="22" t="inlineStr">
-        <is>
-          <t>Cantidad</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="n">
-        <v>93</v>
-      </c>
-      <c r="C20" s="8" t="n">
-        <v>98</v>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>112</v>
-      </c>
-      <c r="E20" s="8" t="n">
-        <v>118</v>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>106</v>
-      </c>
-      <c r="G20" s="8" t="n">
-        <v>112</v>
-      </c>
-      <c r="H20" s="7" t="n">
-        <v>53</v>
-      </c>
-      <c r="I20" s="8" t="n">
-        <v>56</v>
-      </c>
-      <c r="J20" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="K20" s="8" t="n">
-        <v>21</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>890</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1024</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL color</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="n">
-        <v>384</v>
-      </c>
-      <c r="C21" s="10" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL GENERAL</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="n">
-        <v>1280</v>
-      </c>
-      <c r="C23" s="10" t="n">
-        <v>1350</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>Resumen por color (Mín / Máx):</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Negro</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>512</v>
-      </c>
-      <c r="C26" t="n">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Vinotinto</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>384</v>
-      </c>
-      <c r="C27" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Verde Militar</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>384</v>
-      </c>
-      <c r="C28" t="n">
-        <v>405</v>
+      <c r="B21" t="n">
+        <v>299</v>
+      </c>
+      <c r="C21" t="n">
+        <v>389</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B12:C12"/>
+  <mergeCells count="13">
     <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="H12:I12"/>
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J12:K12"/>
     <mergeCell ref="J6:K6"/>
-    <mergeCell ref="A5:L5"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="A17:L17"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:K12"/>
     <mergeCell ref="A11:L11"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B12:C12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2867,7 +2736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2884,14 +2753,14 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>CHAQUETA LITE — COMPRA DE TELA VIORI POR COLOR</t>
+          <t>CHAQUETA LITE — USO TELA DISPONIBLE POR COLOR</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Consumo ficha técnica DAMA · 3 colores 40/30/30 · SS tela +20%</t>
+          <t>Pool global Negro 2500 m · Verde 950 m (Chaqueta + Pant)</t>
         </is>
       </c>
     </row>
@@ -2955,425 +2824,355 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>512</v>
+        <v>890</v>
       </c>
       <c r="D5" t="n">
-        <v>540</v>
+        <v>1024</v>
       </c>
       <c r="E5" t="n">
-        <v>641.34</v>
+        <v>1114.75</v>
       </c>
       <c r="F5" t="n">
-        <v>676.39</v>
+        <v>1282.56</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>769.61</v>
+        <v>1114.75</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>811.67</v>
+        <v>1282.56</v>
       </c>
       <c r="I5" s="23" t="n">
-        <v>82.777</v>
+        <v>119.9</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>87.301</v>
+        <v>137.949</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>Vinotinto</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>384</v>
+        <v>299</v>
       </c>
       <c r="D6" t="n">
-        <v>405</v>
+        <v>389</v>
       </c>
       <c r="E6" t="n">
-        <v>481.01</v>
+        <v>374.44</v>
       </c>
       <c r="F6" t="n">
-        <v>507.33</v>
+        <v>487.32</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>577.21</v>
+        <v>374.44</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>608.8</v>
+        <v>487.32</v>
       </c>
       <c r="I6" s="23" t="n">
-        <v>62.083</v>
+        <v>40.274</v>
       </c>
       <c r="J6" s="24" t="n">
-        <v>65.48</v>
+        <v>52.415</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL TELA VIORI</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1189</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1413</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1489.19</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1769.88</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>1489.19</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>1769.88</v>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>160.174</v>
+      </c>
+      <c r="J7" s="10" t="n">
+        <v>190.364</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>── DETALLE POR TALLA Y COLOR (MÁX) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Color / Talla</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Mts consumo</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Mts compra (+SS)</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Kg compra (+SS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>248</v>
+      </c>
+      <c r="C11" t="n">
+        <v>299</v>
+      </c>
+      <c r="D11" t="n">
+        <v>284</v>
+      </c>
+      <c r="E11" t="n">
+        <v>141</v>
+      </c>
+      <c r="F11" t="n">
+        <v>52</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1024</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1282.56</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>1282.56</v>
+      </c>
+      <c r="J11" t="n">
+        <v>137.949</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>Verde Militar</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>384</v>
-      </c>
-      <c r="D7" t="n">
-        <v>405</v>
-      </c>
-      <c r="E7" t="n">
-        <v>481.01</v>
-      </c>
-      <c r="F7" t="n">
-        <v>507.33</v>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>577.21</v>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>608.8</v>
-      </c>
-      <c r="I7" s="23" t="n">
-        <v>62.083</v>
-      </c>
-      <c r="J7" s="24" t="n">
-        <v>65.48</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL TELA VIORI</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>1280</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1350</v>
-      </c>
-      <c r="E8" t="n">
-        <v>1603.36</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1691.05</v>
-      </c>
-      <c r="G8" s="10" t="n">
-        <v>1924.03</v>
-      </c>
-      <c r="H8" s="10" t="n">
-        <v>2029.26</v>
-      </c>
-      <c r="I8" s="10" t="n">
-        <v>206.944</v>
-      </c>
-      <c r="J8" s="10" t="n">
-        <v>218.262</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>── DETALLE POR TALLA Y COLOR (MÁX) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Color / Talla</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" t="n">
+        <v>94</v>
+      </c>
+      <c r="C12" t="n">
+        <v>113</v>
+      </c>
+      <c r="D12" t="n">
+        <v>108</v>
+      </c>
+      <c r="E12" t="n">
+        <v>54</v>
+      </c>
+      <c r="F12" t="n">
+        <v>20</v>
+      </c>
+      <c r="G12" t="n">
+        <v>389</v>
+      </c>
+      <c r="H12" t="n">
+        <v>487.32</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>487.32</v>
+      </c>
+      <c r="J12" t="n">
+        <v>52.415</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>── CONSUMO UNITARIO VIORI (referencia ficha) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Mts consumo</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Mts compra (+SS)</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>Kg compra (+SS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="27" t="inlineStr">
-        <is>
-          <t>Negro</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>131</v>
-      </c>
-      <c r="C12" t="n">
-        <v>157</v>
-      </c>
-      <c r="D12" t="n">
-        <v>150</v>
-      </c>
-      <c r="E12" t="n">
-        <v>74</v>
-      </c>
-      <c r="F12" t="n">
-        <v>28</v>
-      </c>
-      <c r="G12" t="n">
-        <v>540</v>
-      </c>
-      <c r="H12" t="n">
-        <v>676.39</v>
-      </c>
-      <c r="I12" s="8" t="n">
-        <v>811.67</v>
-      </c>
-      <c r="J12" t="n">
-        <v>87.301</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="29" t="inlineStr">
-        <is>
-          <t>Vinotinto</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>98</v>
-      </c>
-      <c r="C13" t="n">
-        <v>118</v>
-      </c>
-      <c r="D13" t="n">
-        <v>112</v>
-      </c>
-      <c r="E13" t="n">
-        <v>56</v>
-      </c>
-      <c r="F13" t="n">
-        <v>21</v>
-      </c>
-      <c r="G13" t="n">
-        <v>405</v>
-      </c>
-      <c r="H13" t="n">
-        <v>507.33</v>
-      </c>
-      <c r="I13" s="8" t="n">
-        <v>608.8</v>
-      </c>
-      <c r="J13" t="n">
-        <v>65.48</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>Verde Militar</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>98</v>
-      </c>
-      <c r="C14" t="n">
-        <v>118</v>
-      </c>
-      <c r="D14" t="n">
-        <v>112</v>
-      </c>
-      <c r="E14" t="n">
-        <v>56</v>
-      </c>
-      <c r="F14" t="n">
-        <v>21</v>
-      </c>
-      <c r="G14" t="n">
-        <v>405</v>
-      </c>
-      <c r="H14" t="n">
-        <v>507.33</v>
-      </c>
-      <c r="I14" s="8" t="n">
-        <v>608.8</v>
-      </c>
-      <c r="J14" t="n">
-        <v>65.48</v>
-      </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>── CONSUMO UNITARIO VIORI (referencia ficha) ──</t>
-        </is>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Metros/pieza</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1.35</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr">
-        <is>
-          <t>Talla</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>XS</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Metros/pieza</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="C18" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="D18" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="E18" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="F18" t="n">
-        <v>1.35</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Kg/pieza</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.138</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.145</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Kg/pieza</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>0.128</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0.131</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.138</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.144</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.145</v>
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>── OTROS INSUMOS (total producción Mín / Máx) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Elástica 4.5 cm (metros)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>588.11</v>
+      </c>
+      <c r="C20" t="n">
+        <v>698.89</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>── OTROS INSUMOS (total producción Mín / Máx) ──</t>
-        </is>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sesgo cintura 2 cm (metros)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>635.67</v>
+      </c>
+      <c r="C21" t="n">
+        <v>755.41</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Elástica 4.5 cm (metros)</t>
+          <t>Sesgo manga 2 cm (metros)</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>633.15</v>
+        <v>231.41</v>
       </c>
       <c r="C22" t="n">
-        <v>667.76</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Sesgo cintura 2 cm (metros)</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>684.35</v>
-      </c>
-      <c r="C23" t="n">
-        <v>721.76</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Sesgo manga 2 cm (metros)</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>249.15</v>
-      </c>
-      <c r="C24" t="n">
-        <v>262.76</v>
+        <v>274.99</v>
       </c>
     </row>
   </sheetData>
@@ -3414,7 +3213,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="31" t="inlineStr">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>★ = tienda con velocidad proyectada/ajustada</t>
         </is>
@@ -3511,34 +3310,34 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C5" s="24" t="n">
+        <v>59</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>60</v>
+      </c>
+      <c r="E5" s="24" t="n">
+        <v>71</v>
+      </c>
+      <c r="F5" s="23" t="n">
         <v>57</v>
       </c>
-      <c r="D5" s="23" t="n">
-        <v>64</v>
-      </c>
-      <c r="E5" s="24" t="n">
+      <c r="G5" s="24" t="n">
         <v>68</v>
       </c>
-      <c r="F5" s="23" t="n">
-        <v>61</v>
-      </c>
-      <c r="G5" s="24" t="n">
-        <v>65</v>
-      </c>
       <c r="H5" s="23" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J5" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="K5" s="24" t="n">
         <v>12</v>
-      </c>
-      <c r="K5" s="24" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -3548,28 +3347,28 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C6" s="24" t="n">
+        <v>39</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>39</v>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>46</v>
+      </c>
+      <c r="F6" s="23" t="n">
         <v>37</v>
       </c>
-      <c r="D6" s="23" t="n">
-        <v>42</v>
-      </c>
-      <c r="E6" s="24" t="n">
+      <c r="G6" s="24" t="n">
         <v>44</v>
       </c>
-      <c r="F6" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="G6" s="24" t="n">
-        <v>42</v>
-      </c>
       <c r="H6" s="23" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I6" s="24" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J6" s="23" t="n">
         <v>7</v>
@@ -3585,34 +3384,34 @@
         </is>
       </c>
       <c r="B7" s="23" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C7" s="24" t="n">
+        <v>39</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="E7" s="24" t="n">
+        <v>47</v>
+      </c>
+      <c r="F7" s="23" t="n">
         <v>38</v>
       </c>
-      <c r="D7" s="23" t="n">
-        <v>43</v>
-      </c>
-      <c r="E7" s="24" t="n">
+      <c r="G7" s="24" t="n">
         <v>45</v>
       </c>
-      <c r="F7" s="23" t="n">
-        <v>41</v>
-      </c>
-      <c r="G7" s="24" t="n">
-        <v>43</v>
-      </c>
       <c r="H7" s="23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I7" s="24" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K7" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -3622,28 +3421,28 @@
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C8" s="24" t="n">
+        <v>45</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>54</v>
+      </c>
+      <c r="F8" s="23" t="n">
         <v>43</v>
       </c>
-      <c r="D8" s="23" t="n">
-        <v>49</v>
-      </c>
-      <c r="E8" s="24" t="n">
-        <v>52</v>
-      </c>
-      <c r="F8" s="23" t="n">
-        <v>47</v>
-      </c>
       <c r="G8" s="24" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="J8" s="23" t="n">
         <v>8</v>
@@ -3653,7 +3452,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>GRAND PLAZ ★</t>
         </is>
@@ -3662,13 +3461,13 @@
         <v>8</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D9" s="23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E9" s="24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F9" s="23" t="n">
         <v>9</v>
@@ -3677,7 +3476,7 @@
         <v>10</v>
       </c>
       <c r="H9" s="23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I9" s="24" t="n">
         <v>5</v>
@@ -3690,145 +3489,145 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>LA VELA ★</t>
         </is>
       </c>
       <c r="B10" s="23" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C10" s="24" t="n">
+        <v>49</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="E10" s="24" t="n">
+        <v>59</v>
+      </c>
+      <c r="F10" s="23" t="n">
         <v>47</v>
       </c>
-      <c r="D10" s="23" t="n">
-        <v>54</v>
-      </c>
-      <c r="E10" s="24" t="n">
-        <v>57</v>
-      </c>
-      <c r="F10" s="23" t="n">
-        <v>51</v>
-      </c>
       <c r="G10" s="24" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I10" s="24" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J10" s="23" t="n">
         <v>9</v>
       </c>
       <c r="K10" s="24" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="32" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>TOLON ★</t>
         </is>
       </c>
       <c r="B11" s="23" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C11" s="24" t="n">
+        <v>38</v>
+      </c>
+      <c r="D11" s="23" t="n">
+        <v>39</v>
+      </c>
+      <c r="E11" s="24" t="n">
+        <v>46</v>
+      </c>
+      <c r="F11" s="23" t="n">
         <v>37</v>
       </c>
-      <c r="D11" s="23" t="n">
-        <v>42</v>
-      </c>
-      <c r="E11" s="24" t="n">
+      <c r="G11" s="24" t="n">
         <v>44</v>
       </c>
-      <c r="F11" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="G11" s="24" t="n">
-        <v>42</v>
-      </c>
       <c r="H11" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="I11" s="24" t="n">
+        <v>22</v>
+      </c>
+      <c r="J11" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="K11" s="24" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="31" t="inlineStr">
+        <is>
+          <t>WEB ★</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="I11" s="24" t="n">
-        <v>21</v>
-      </c>
-      <c r="J11" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="K11" s="24" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="32" t="inlineStr">
-        <is>
-          <t>WEB ★</t>
-        </is>
-      </c>
-      <c r="B12" s="23" t="n">
-        <v>21</v>
-      </c>
       <c r="C12" s="24" t="n">
+        <v>24</v>
+      </c>
+      <c r="D12" s="23" t="n">
+        <v>24</v>
+      </c>
+      <c r="E12" s="24" t="n">
+        <v>28</v>
+      </c>
+      <c r="F12" s="23" t="n">
         <v>23</v>
       </c>
-      <c r="D12" s="23" t="n">
-        <v>26</v>
-      </c>
-      <c r="E12" s="24" t="n">
+      <c r="G12" s="24" t="n">
         <v>27</v>
       </c>
-      <c r="F12" s="23" t="n">
-        <v>24</v>
-      </c>
-      <c r="G12" s="24" t="n">
-        <v>26</v>
-      </c>
       <c r="H12" s="23" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I12" s="24" t="n">
         <v>13</v>
       </c>
       <c r="J12" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="K12" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="K12" s="24" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="13">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>BARQUISIMETO ★</t>
         </is>
       </c>
       <c r="B13" s="23" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C13" s="24" t="n">
+        <v>41</v>
+      </c>
+      <c r="D13" s="23" t="n">
+        <v>41</v>
+      </c>
+      <c r="E13" s="24" t="n">
+        <v>49</v>
+      </c>
+      <c r="F13" s="23" t="n">
         <v>39</v>
       </c>
-      <c r="D13" s="23" t="n">
-        <v>44</v>
-      </c>
-      <c r="E13" s="24" t="n">
+      <c r="G13" s="24" t="n">
         <v>47</v>
       </c>
-      <c r="F13" s="23" t="n">
-        <v>42</v>
-      </c>
-      <c r="G13" s="24" t="n">
-        <v>44</v>
-      </c>
       <c r="H13" s="23" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I13" s="24" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J13" s="23" t="n">
         <v>8</v>
@@ -3844,34 +3643,34 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>312</v>
+        <v>289</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>329</v>
+        <v>343</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>374</v>
+        <v>347</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>394</v>
+        <v>411</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>355</v>
+        <v>330</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>375</v>
+        <v>392</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16">
@@ -3910,10 +3709,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="C18" t="n">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="D18" t="n">
         <v>93.3</v>
@@ -3926,10 +3725,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="C19" t="n">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="D19" t="n">
         <v>61</v>
@@ -3942,10 +3741,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="C20" t="n">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="D20" t="n">
         <v>62.1</v>
@@ -3958,10 +3757,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="C21" t="n">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="D21" t="n">
         <v>71</v>
@@ -3974,10 +3773,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C22" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D22" t="n">
         <v>14</v>
@@ -3990,10 +3789,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>184</v>
+        <v>171</v>
       </c>
       <c r="C23" t="n">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="D23" t="n">
         <v>77.7</v>
@@ -4006,10 +3805,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C24" t="n">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="D24" t="n">
         <v>60.4</v>
@@ -4022,10 +3821,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C25" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D25" t="n">
         <v>37.2</v>
@@ -4038,10 +3837,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="C26" t="n">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D26" t="n">
         <v>64.09999999999999</v>
@@ -4073,7 +3872,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="33" t="inlineStr">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>PLAN DE CIERRES — QX NEGRO 0580 (INVENTARIO GLOBAL)</t>
         </is>
@@ -4225,10 +4024,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1038</v>
+        <v>965</v>
       </c>
       <c r="D14" t="n">
-        <v>1095</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="15">
@@ -4243,10 +4042,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>242</v>
+        <v>224</v>
       </c>
       <c r="D15" t="n">
-        <v>255</v>
+        <v>266</v>
       </c>
     </row>
     <row r="16">
@@ -4257,16 +4056,16 @@
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>1280</v>
+        <v>1189</v>
       </c>
       <c r="D16" t="n">
-        <v>1350</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>── ASIGNACIÓN AL MÁXIMO (1350 und) ──</t>
+          <t>── ASIGNACIÓN AL MÁXIMO (1413 und) ──</t>
         </is>
       </c>
     </row>
@@ -4299,7 +4098,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>347</v>
+        <v>399</v>
       </c>
     </row>
     <row r="22">
@@ -4309,7 +4108,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>255</v>
+        <v>266</v>
       </c>
     </row>
     <row r="23">
@@ -4319,7 +4118,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>602</v>
+        <v>665</v>
       </c>
     </row>
     <row r="24">
@@ -4329,7 +4128,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1350</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="25">
@@ -4339,7 +4138,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>142</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27">
@@ -4350,7 +4149,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1280 – 1350 und</t>
+          <t>1189 – 1413 und</t>
         </is>
       </c>
     </row>
@@ -4384,7 +4183,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="34" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>METODOLOGÍA — PROYECCIÓN CHAQUETA LITE</t>
         </is>
@@ -4614,7 +4413,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Al máximo (1350 und) quedan 142 cierres remanentes.</t>
+          <t xml:space="preserve">   Al máximo (1413 und) quedan 79 cierres remanentes.</t>
         </is>
       </c>
     </row>
@@ -4631,14 +4430,14 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Compromiso mín: 1280 und.</t>
+          <t xml:space="preserve">   Compromiso mín: 1189 und.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Techo máx: 1350 und.</t>
+          <t xml:space="preserve">   Techo máx: 1413 und.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Curva tallas: refuerzo moderado núcleo S+M en chaqueta y pant
+0,75 pp a S y M (igual en ambos modelos), descuento proporcional XS/L/XL
sobre base analítica Jacket / Basic Line; Excel regenerados con tela real

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -637,7 +637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1.2525</v>
+        <v>1.2524</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1347,45 +1347,47 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>XL 5.1%</t>
+          <t>XL 4.9%</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>hist XL 3.6% · L 13.8% · XS sin cambio</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+          <t>hist XL 3.6% · L 13.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Núcleo S+M (+0.75 pp c/u)</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>S 29.9% · M 28.5%</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Descuento proporcional XS/L/XL · criterio I+D</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Tolón histórico</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Tolón proyectado (85% Chacao)</t>
+          <t>Tolón histórico</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>60.4</v>
+        <v>8.1</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1396,11 +1398,11 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Web histórica</t>
+          <t>Tolón proyectado (85% Chacao)</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>7.8</v>
+        <v>60.4</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1411,11 +1413,11 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Web proyectada (60% Cerro Verde)</t>
+          <t>Web histórica</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>37.2</v>
+        <v>7.8</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1426,11 +1428,11 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>La Vela histórica</t>
+          <t>Web proyectada (60% Cerro Verde)</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>10</v>
+        <v>37.2</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1441,11 +1443,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+          <t>La Vela histórica</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>77.7</v>
+        <v>10</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1456,11 +1458,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Grand Plaz histórica</t>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>8.300000000000001</v>
+        <v>77.7</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1471,11 +1473,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+68% hist.)</t>
+          <t>Grand Plaz histórica</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>14</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -1486,11 +1488,11 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+          <t>Grand Plaz proyectada (+68% hist.)</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>64.09999999999999</v>
+        <v>14</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -1501,45 +1503,60 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>Corporativo</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>EXCLUIDO</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
+        <is>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
         <is>
           <t>• Preferencia: 60 cm → XS/S/M · 75 cm → L/XL · excedente 75 cm adaptable a 60 cm.</t>
         </is>
@@ -1627,23 +1644,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>24.3%</t>
+          <t>23.4%</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>60</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="F5" t="n">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="G5" t="n">
-        <v>343</v>
+        <v>331</v>
       </c>
     </row>
     <row r="6">
@@ -1654,23 +1671,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>29.2%</t>
+          <t>29.9%</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>60</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>347</v>
+        <v>356</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>412</v>
+        <v>423</v>
       </c>
       <c r="F6" t="n">
-        <v>347</v>
+        <v>356</v>
       </c>
       <c r="G6" t="n">
-        <v>412</v>
+        <v>423</v>
       </c>
     </row>
     <row r="7">
@@ -1681,23 +1698,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>27.7%</t>
+          <t>28.5%</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>60</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>330</v>
+        <v>339</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>392</v>
+        <v>402</v>
       </c>
       <c r="F7" t="n">
-        <v>330</v>
+        <v>339</v>
       </c>
       <c r="G7" t="n">
-        <v>392</v>
+        <v>402</v>
       </c>
     </row>
     <row r="8">
@@ -1708,23 +1725,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.8%</t>
+          <t>13.3%</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>75</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="F8" t="n">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="G8" t="n">
-        <v>195</v>
+        <v>188</v>
       </c>
     </row>
     <row r="9">
@@ -1735,23 +1752,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>5.1%</t>
+          <t>4.9%</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>75</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F9" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G9" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10">
@@ -1767,10 +1784,10 @@
         <v>1413</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>965</v>
+        <v>973</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>1147</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="12">
@@ -1799,7 +1816,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Incl. 399 cierres 75→60 cm</t>
+          <t>Incl. 408 cierres 75→60 cm</t>
         </is>
       </c>
     </row>
@@ -1899,16 +1916,16 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="F7" s="18" t="n">
         <v>45</v>
@@ -1924,16 +1941,16 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F8" s="18" t="n">
         <v>15</v>
@@ -1949,16 +1966,16 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="C9" s="20" t="n">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="D9" s="20" t="n">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="F9" s="20" t="n">
         <v>60</v>
@@ -2018,19 +2035,19 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="E13" s="18" t="n">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>1024</v>
@@ -2043,19 +2060,19 @@
         </is>
       </c>
       <c r="B14" s="18" t="n">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C14" s="18" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D14" s="18" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G14" s="18" t="n">
         <v>389</v>
@@ -2068,19 +2085,19 @@
         </is>
       </c>
       <c r="B15" s="20" t="n">
-        <v>342</v>
+        <v>331</v>
       </c>
       <c r="C15" s="20" t="n">
-        <v>412</v>
+        <v>422</v>
       </c>
       <c r="D15" s="20" t="n">
-        <v>392</v>
+        <v>403</v>
       </c>
       <c r="E15" s="20" t="n">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="F15" s="20" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="G15" s="20" t="n">
         <v>1413</v>
@@ -2130,7 +2147,7 @@
         <v>1114.75</v>
       </c>
       <c r="C19" s="24" t="n">
-        <v>1282.56</v>
+        <v>1282.42</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2150,10 +2167,10 @@
         </is>
       </c>
       <c r="B20" s="23" t="n">
-        <v>374.44</v>
+        <v>374.53</v>
       </c>
       <c r="C20" s="24" t="n">
-        <v>487.32</v>
+        <v>487.22</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2173,10 +2190,10 @@
         </is>
       </c>
       <c r="B21" s="23" t="n">
-        <v>1489.19</v>
+        <v>1489.28</v>
       </c>
       <c r="C21" s="24" t="n">
-        <v>1769.88</v>
+        <v>1769.64</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2185,7 +2202,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>190.364 kg al máx · consumo = tela disponible</t>
+          <t>190.341 kg al máx · consumo = tela disponible</t>
         </is>
       </c>
     </row>
@@ -2196,10 +2213,10 @@
         </is>
       </c>
       <c r="B22" s="23" t="n">
-        <v>588.11</v>
+        <v>588.12</v>
       </c>
       <c r="C22" s="24" t="n">
-        <v>698.89</v>
+        <v>698.91</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2219,10 +2236,10 @@
         </is>
       </c>
       <c r="B23" s="23" t="n">
-        <v>635.67</v>
+        <v>635.6799999999999</v>
       </c>
       <c r="C23" s="24" t="n">
-        <v>755.41</v>
+        <v>755.4299999999999</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2242,10 +2259,10 @@
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>231.41</v>
+        <v>231.42</v>
       </c>
       <c r="C24" s="24" t="n">
-        <v>274.99</v>
+        <v>275.01</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2288,10 +2305,10 @@
         </is>
       </c>
       <c r="B26" s="26" t="n">
-        <v>965</v>
+        <v>973</v>
       </c>
       <c r="C26" s="26" t="n">
-        <v>1147</v>
+        <v>1156</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2311,10 +2328,10 @@
         </is>
       </c>
       <c r="B27" s="26" t="n">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C27" s="26" t="n">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2480,34 +2497,34 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>45</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
@@ -2621,34 +2638,34 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>15</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
@@ -2837,19 +2854,19 @@
         <v>1114.75</v>
       </c>
       <c r="F5" t="n">
-        <v>1282.56</v>
+        <v>1282.42</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>1114.75</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>1282.56</v>
+        <v>1282.42</v>
       </c>
       <c r="I5" s="23" t="n">
-        <v>119.9</v>
+        <v>119.901</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>137.949</v>
+        <v>137.936</v>
       </c>
     </row>
     <row r="6">
@@ -2870,22 +2887,22 @@
         <v>389</v>
       </c>
       <c r="E6" t="n">
-        <v>374.44</v>
+        <v>374.53</v>
       </c>
       <c r="F6" t="n">
-        <v>487.32</v>
+        <v>487.22</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>374.44</v>
+        <v>374.53</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>487.32</v>
+        <v>487.22</v>
       </c>
       <c r="I6" s="23" t="n">
-        <v>40.274</v>
+        <v>40.284</v>
       </c>
       <c r="J6" s="24" t="n">
-        <v>52.415</v>
+        <v>52.405</v>
       </c>
     </row>
     <row r="7">
@@ -2901,22 +2918,22 @@
         <v>1413</v>
       </c>
       <c r="E7" t="n">
-        <v>1489.19</v>
+        <v>1489.28</v>
       </c>
       <c r="F7" t="n">
-        <v>1769.88</v>
+        <v>1769.64</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>1489.19</v>
+        <v>1489.28</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>1769.88</v>
+        <v>1769.64</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>160.174</v>
+        <v>160.185</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>190.364</v>
+        <v>190.341</v>
       </c>
     </row>
     <row r="9">
@@ -2985,31 +3002,31 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="C11" t="n">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="D11" t="n">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="E11" t="n">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="F11" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G11" t="n">
         <v>1024</v>
       </c>
       <c r="H11" t="n">
-        <v>1282.56</v>
+        <v>1282.42</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>1282.56</v>
+        <v>1282.42</v>
       </c>
       <c r="J11" t="n">
-        <v>137.949</v>
+        <v>137.936</v>
       </c>
     </row>
     <row r="12">
@@ -3019,31 +3036,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C12" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D12" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E12" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F12" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G12" t="n">
         <v>389</v>
       </c>
       <c r="H12" t="n">
-        <v>487.32</v>
+        <v>487.22</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>487.32</v>
+        <v>487.22</v>
       </c>
       <c r="J12" t="n">
-        <v>52.415</v>
+        <v>52.405</v>
       </c>
     </row>
     <row r="14">
@@ -3143,10 +3160,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>588.11</v>
+        <v>588.12</v>
       </c>
       <c r="C20" t="n">
-        <v>698.89</v>
+        <v>698.91</v>
       </c>
     </row>
     <row r="21">
@@ -3156,10 +3173,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>635.67</v>
+        <v>635.6799999999999</v>
       </c>
       <c r="C21" t="n">
-        <v>755.41</v>
+        <v>755.4299999999999</v>
       </c>
     </row>
     <row r="22">
@@ -3169,10 +3186,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>231.41</v>
+        <v>231.42</v>
       </c>
       <c r="C22" t="n">
-        <v>274.99</v>
+        <v>275.01</v>
       </c>
     </row>
   </sheetData>
@@ -3310,34 +3327,34 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C5" s="24" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D5" s="23" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E5" s="24" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H5" s="23" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J5" s="23" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K5" s="24" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -3347,28 +3364,28 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D6" s="23" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H6" s="23" t="n">
         <v>18</v>
       </c>
       <c r="I6" s="24" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J6" s="23" t="n">
         <v>7</v>
@@ -3384,25 +3401,25 @@
         </is>
       </c>
       <c r="B7" s="23" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C7" s="24" t="n">
+        <v>38</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>41</v>
+      </c>
+      <c r="E7" s="24" t="n">
+        <v>48</v>
+      </c>
+      <c r="F7" s="23" t="n">
         <v>39</v>
       </c>
-      <c r="D7" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="E7" s="24" t="n">
-        <v>47</v>
-      </c>
-      <c r="F7" s="23" t="n">
-        <v>38</v>
-      </c>
       <c r="G7" s="24" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H7" s="23" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I7" s="24" t="n">
         <v>22</v>
@@ -3411,7 +3428,7 @@
         <v>6</v>
       </c>
       <c r="K7" s="24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -3421,31 +3438,31 @@
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" s="24" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F8" s="23" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J8" s="23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K8" s="24" t="n">
         <v>9</v>
@@ -3458,7 +3475,7 @@
         </is>
       </c>
       <c r="B9" s="23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>9</v>
@@ -3473,7 +3490,7 @@
         <v>9</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H9" s="23" t="n">
         <v>4</v>
@@ -3482,10 +3499,10 @@
         <v>5</v>
       </c>
       <c r="J9" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="24" t="n">
         <v>1</v>
-      </c>
-      <c r="K9" s="24" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -3495,34 +3512,34 @@
         </is>
       </c>
       <c r="B10" s="23" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C10" s="24" t="n">
+        <v>48</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>51</v>
+      </c>
+      <c r="E10" s="24" t="n">
+        <v>61</v>
+      </c>
+      <c r="F10" s="23" t="n">
         <v>49</v>
       </c>
-      <c r="D10" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="E10" s="24" t="n">
-        <v>59</v>
-      </c>
-      <c r="F10" s="23" t="n">
-        <v>47</v>
-      </c>
       <c r="G10" s="24" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I10" s="24" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J10" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="K10" s="24" t="n">
         <v>9</v>
-      </c>
-      <c r="K10" s="24" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -3532,31 +3549,31 @@
         </is>
       </c>
       <c r="B11" s="23" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="24" t="n">
+        <v>37</v>
+      </c>
+      <c r="D11" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="E11" s="24" t="n">
+        <v>47</v>
+      </c>
+      <c r="F11" s="23" t="n">
         <v>38</v>
       </c>
-      <c r="D11" s="23" t="n">
-        <v>39</v>
-      </c>
-      <c r="E11" s="24" t="n">
-        <v>46</v>
-      </c>
-      <c r="F11" s="23" t="n">
-        <v>37</v>
-      </c>
       <c r="G11" s="24" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H11" s="23" t="n">
         <v>18</v>
       </c>
       <c r="I11" s="24" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J11" s="23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K11" s="24" t="n">
         <v>8</v>
@@ -3569,22 +3586,22 @@
         </is>
       </c>
       <c r="B12" s="23" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12" s="24" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E12" s="24" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F12" s="23" t="n">
         <v>23</v>
       </c>
       <c r="G12" s="24" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H12" s="23" t="n">
         <v>11</v>
@@ -3596,7 +3613,7 @@
         <v>4</v>
       </c>
       <c r="K12" s="24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -3606,34 +3623,34 @@
         </is>
       </c>
       <c r="B13" s="23" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C13" s="24" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D13" s="23" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E13" s="24" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F13" s="23" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G13" s="24" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H13" s="23" t="n">
         <v>19</v>
       </c>
       <c r="I13" s="24" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J13" s="23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -3643,34 +3660,34 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>347</v>
+        <v>356</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>411</v>
+        <v>422</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>392</v>
+        <v>403</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16">
@@ -4024,10 +4041,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>965</v>
+        <v>973</v>
       </c>
       <c r="D14" t="n">
-        <v>1147</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="15">
@@ -4042,10 +4059,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="D15" t="n">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16">
@@ -4098,7 +4115,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>399</v>
+        <v>408</v>
       </c>
     </row>
     <row r="22">
@@ -4108,7 +4125,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="23">
@@ -4176,7 +4193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A56"/>
+  <dimension ref="A1:A57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -4461,74 +4478,81 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">   XL reforzado +1.5 pp desde L → L 13.8% · XL 5.1% (XS sin cambio).</t>
+          <t xml:space="preserve">   XL reforzado +1.5 pp desde L → L 13.3% · XL 4.9%.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Núcleo S+M: +0.75 pp a S y a M (igual en chaqueta y pant); resto desde XS/L/XL proporcional.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="13" t="inlineStr">
+      <c r="A47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
         <is>
           <t>8. DISTRIBUCIÓN</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Por talla: curva histórica ajustada (ver sección 7).</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-    </row>
     <row r="51">
-      <c r="A51" s="13" t="inlineStr">
+      <c r="A51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="13" t="inlineStr">
         <is>
           <t>9. COLORES Y COMPRA DE TELA</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Colores: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
+          <t xml:space="preserve">   Colores: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Consumo VIORI por pieza (ficha técnica): XS 1.19m · S 1.22m · M 1.28m · L 1.34m · XL 1.35m.</t>
+          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Stock de seguridad tela: +20% sobre consumo (compra = consumo × 1.2).</t>
+          <t xml:space="preserve">   Consumo VIORI por pieza (ficha técnica): XS 1.19m · S 1.22m · M 1.28m · L 1.34m · XL 1.35m.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Stock de seguridad tela: +20% sobre consumo (compra = consumo × 1.2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
         <is>
           <t xml:space="preserve">   Ver hojas 'Producción Color × Talla' y 'Compra de Tela VIORI'.</t>
         </is>

</xml_diff>

<commit_message>
Curva tallas: XS 20,5% chaqueta y 18% pant; exceso a S y M 50/50
Reemplaza refuerzo genérico S+M; L/XL sin cambio. Excel regenerados.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -1014,7 +1014,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1413</v>
+        <v>1410</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1074,7 +1074,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1413</v>
+        <v>1410</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1.2524</v>
+        <v>1.2548</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1257,11 +1257,11 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>mín · máx 1024 und</t>
+          <t>mín · máx 1022 und</t>
         </is>
       </c>
     </row>
@@ -1272,11 +1272,11 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>mín · máx 389 und</t>
+          <t>mín · máx 388 und</t>
         </is>
       </c>
     </row>
@@ -1347,29 +1347,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>XL 4.9%</t>
+          <t>XL 5.1%</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>hist XL 3.6% · L 13.3%</t>
+          <t>hist XL 3.6% · L 13.8%</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Núcleo S+M (+0.75 pp c/u)</t>
+          <t>XS objetivo 20.5%</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>S 29.9% · M 28.5%</t>
+          <t>XS 20.5%</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Descuento proporcional XS/L/XL · criterio I+D</t>
+          <t>Exceso repartido 50/50 a S y M · L/XL sin cambio</t>
         </is>
       </c>
     </row>
@@ -1644,23 +1644,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>23.4%</t>
+          <t>20.5%</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>60</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>278</v>
+        <v>243</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>331</v>
+        <v>289</v>
       </c>
       <c r="F5" t="n">
-        <v>278</v>
+        <v>243</v>
       </c>
       <c r="G5" t="n">
-        <v>331</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6">
@@ -1671,23 +1671,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>29.9%</t>
+          <t>31.0%</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>60</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>423</v>
+        <v>438</v>
       </c>
       <c r="F6" t="n">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="G6" t="n">
-        <v>423</v>
+        <v>438</v>
       </c>
     </row>
     <row r="7">
@@ -1698,23 +1698,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>28.5%</t>
+          <t>29.6%</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>60</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>402</v>
+        <v>417</v>
       </c>
       <c r="F7" t="n">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="G7" t="n">
-        <v>402</v>
+        <v>417</v>
       </c>
     </row>
     <row r="8">
@@ -1725,23 +1725,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.3%</t>
+          <t>13.8%</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>75</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="F8" t="n">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="G8" t="n">
-        <v>188</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9">
@@ -1752,23 +1752,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4.9%</t>
+          <t>5.1%</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>75</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F9" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G9" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10">
@@ -1778,16 +1778,16 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>1413</v>
+        <v>1410</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>973</v>
+        <v>962</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>1156</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="12">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Usa máx 1413 (95%)</t>
+          <t>Usa máx 1410 (95%)</t>
         </is>
       </c>
     </row>
@@ -1812,11 +1812,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Incl. 408 cierres 75→60 cm</t>
+          <t>Incl. 396 cierres 75→60 cm</t>
         </is>
       </c>
     </row>
@@ -1861,14 +1861,14 @@
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Rango producción: 1189 – 1413 und</t>
+          <t>Rango producción: 1187 – 1410 und</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>MÍNIMO — 1189 und (compromiso)</t>
+          <t>MÍNIMO — 1187 und (compromiso)</t>
         </is>
       </c>
     </row>
@@ -1916,22 +1916,22 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>208</v>
+        <v>182</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="F7" s="18" t="n">
         <v>45</v>
       </c>
       <c r="G7" s="18" t="n">
-        <v>890</v>
+        <v>889</v>
       </c>
     </row>
     <row r="8">
@@ -1941,22 +1941,22 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G8" s="18" t="n">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9">
@@ -1966,28 +1966,28 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>278</v>
+        <v>243</v>
       </c>
       <c r="C9" s="20" t="n">
-        <v>355</v>
+        <v>368</v>
       </c>
       <c r="D9" s="20" t="n">
-        <v>338</v>
+        <v>351</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G9" s="20" t="n">
-        <v>1189</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>MÁXIMO — 1413 und (techo)</t>
+          <t>MÁXIMO — 1410 und (techo)</t>
         </is>
       </c>
     </row>
@@ -2035,22 +2035,22 @@
         </is>
       </c>
       <c r="B13" s="18" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C13" s="18" t="n">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="E13" s="18" t="n">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G13" s="18" t="n">
-        <v>1024</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="14">
@@ -2060,22 +2060,22 @@
         </is>
       </c>
       <c r="B14" s="18" t="n">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="C14" s="18" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D14" s="18" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F14" s="18" t="n">
         <v>19</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="15">
@@ -2085,22 +2085,22 @@
         </is>
       </c>
       <c r="B15" s="20" t="n">
-        <v>331</v>
+        <v>290</v>
       </c>
       <c r="C15" s="20" t="n">
-        <v>422</v>
+        <v>437</v>
       </c>
       <c r="D15" s="20" t="n">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="E15" s="20" t="n">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="F15" s="20" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G15" s="20" t="n">
-        <v>1413</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="17">
@@ -2144,10 +2144,10 @@
         </is>
       </c>
       <c r="B19" s="23" t="n">
-        <v>1114.75</v>
+        <v>1115.51</v>
       </c>
       <c r="C19" s="24" t="n">
-        <v>1282.42</v>
+        <v>1282.27</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2167,10 +2167,10 @@
         </is>
       </c>
       <c r="B20" s="23" t="n">
-        <v>374.53</v>
+        <v>374.01</v>
       </c>
       <c r="C20" s="24" t="n">
-        <v>487.22</v>
+        <v>486.81</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2190,10 +2190,10 @@
         </is>
       </c>
       <c r="B21" s="23" t="n">
-        <v>1489.28</v>
+        <v>1489.52</v>
       </c>
       <c r="C21" s="24" t="n">
-        <v>1769.64</v>
+        <v>1769.08</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>190.341 kg al máx · consumo = tela disponible</t>
+          <t>190.281 kg al máx · consumo = tela disponible</t>
         </is>
       </c>
     </row>
@@ -2213,10 +2213,10 @@
         </is>
       </c>
       <c r="B22" s="23" t="n">
-        <v>588.12</v>
+        <v>587.8200000000001</v>
       </c>
       <c r="C22" s="24" t="n">
-        <v>698.91</v>
+        <v>698.22</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2236,10 +2236,10 @@
         </is>
       </c>
       <c r="B23" s="23" t="n">
-        <v>635.6799999999999</v>
+        <v>635.3</v>
       </c>
       <c r="C23" s="24" t="n">
-        <v>755.4299999999999</v>
+        <v>754.62</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2259,10 +2259,10 @@
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>231.42</v>
+        <v>231.72</v>
       </c>
       <c r="C24" s="24" t="n">
-        <v>275.01</v>
+        <v>275.22</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2282,10 +2282,10 @@
         </is>
       </c>
       <c r="B25" s="23" t="n">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="C25" s="24" t="n">
-        <v>1413</v>
+        <v>1410</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Pool global 1492 und · rem. 79 al máx</t>
+          <t>Pool global 1492 und · rem. 82 al máx</t>
         </is>
       </c>
     </row>
@@ -2305,10 +2305,10 @@
         </is>
       </c>
       <c r="B26" s="26" t="n">
-        <v>973</v>
+        <v>962</v>
       </c>
       <c r="C26" s="26" t="n">
-        <v>1156</v>
+        <v>1144</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2328,10 +2328,10 @@
         </is>
       </c>
       <c r="B27" s="26" t="n">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="C27" s="26" t="n">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2395,14 +2395,14 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Rango global: 1189 – 1413 und</t>
+          <t>Rango global: 1187 – 1410 und</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>Negro (1024 und máx)</t>
+          <t>Negro (1022 und máx)</t>
         </is>
       </c>
     </row>
@@ -2497,34 +2497,34 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>208</v>
+        <v>182</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>266</v>
+        <v>276</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="J8" s="7" t="n">
         <v>45</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9">
@@ -2534,16 +2534,16 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>1024</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
         <is>
-          <t>Verde Militar (389 und máx)</t>
+          <t>Verde Militar (388 und máx)</t>
         </is>
       </c>
     </row>
@@ -2638,31 +2638,31 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K14" s="8" t="n">
         <v>19</v>
@@ -2675,10 +2675,10 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="17">
@@ -2688,10 +2688,10 @@
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="C17" s="10" t="n">
-        <v>1413</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="19">
@@ -2708,10 +2708,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="C20" t="n">
-        <v>1024</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="21">
@@ -2721,10 +2721,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C21" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>
@@ -2845,28 +2845,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="D5" t="n">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="E5" t="n">
-        <v>1114.75</v>
+        <v>1115.51</v>
       </c>
       <c r="F5" t="n">
-        <v>1282.42</v>
+        <v>1282.27</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>1114.75</v>
+        <v>1115.51</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>1282.42</v>
+        <v>1282.27</v>
       </c>
       <c r="I5" s="23" t="n">
-        <v>119.901</v>
+        <v>119.983</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>137.936</v>
+        <v>137.92</v>
       </c>
     </row>
     <row r="6">
@@ -2881,28 +2881,28 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D6" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E6" t="n">
-        <v>374.53</v>
+        <v>374.01</v>
       </c>
       <c r="F6" t="n">
-        <v>487.22</v>
+        <v>486.81</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>374.53</v>
+        <v>374.01</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>487.22</v>
+        <v>486.81</v>
       </c>
       <c r="I6" s="23" t="n">
-        <v>40.284</v>
+        <v>40.228</v>
       </c>
       <c r="J6" s="24" t="n">
-        <v>52.405</v>
+        <v>52.361</v>
       </c>
     </row>
     <row r="7">
@@ -2912,28 +2912,28 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="D7" t="n">
-        <v>1413</v>
+        <v>1410</v>
       </c>
       <c r="E7" t="n">
-        <v>1489.28</v>
+        <v>1489.52</v>
       </c>
       <c r="F7" t="n">
-        <v>1769.64</v>
+        <v>1769.08</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>1489.28</v>
+        <v>1489.52</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>1769.64</v>
+        <v>1769.08</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>160.185</v>
+        <v>160.211</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>190.341</v>
+        <v>190.281</v>
       </c>
     </row>
     <row r="9">
@@ -3002,31 +3002,31 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="C11" t="n">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="D11" t="n">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="E11" t="n">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="F11" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G11" t="n">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="H11" t="n">
-        <v>1282.42</v>
+        <v>1282.27</v>
       </c>
       <c r="I11" s="8" t="n">
-        <v>1282.42</v>
+        <v>1282.27</v>
       </c>
       <c r="J11" t="n">
-        <v>137.936</v>
+        <v>137.92</v>
       </c>
     </row>
     <row r="12">
@@ -3036,31 +3036,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="C12" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D12" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E12" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F12" t="n">
         <v>19</v>
       </c>
       <c r="G12" t="n">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H12" t="n">
-        <v>487.22</v>
+        <v>486.81</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>487.22</v>
+        <v>486.81</v>
       </c>
       <c r="J12" t="n">
-        <v>52.405</v>
+        <v>52.361</v>
       </c>
     </row>
     <row r="14">
@@ -3160,10 +3160,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>588.12</v>
+        <v>587.8200000000001</v>
       </c>
       <c r="C20" t="n">
-        <v>698.91</v>
+        <v>698.22</v>
       </c>
     </row>
     <row r="21">
@@ -3173,10 +3173,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>635.6799999999999</v>
+        <v>635.3</v>
       </c>
       <c r="C21" t="n">
-        <v>755.4299999999999</v>
+        <v>754.62</v>
       </c>
     </row>
     <row r="22">
@@ -3186,10 +3186,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>231.42</v>
+        <v>231.72</v>
       </c>
       <c r="C22" t="n">
-        <v>275.01</v>
+        <v>275.22</v>
       </c>
     </row>
   </sheetData>
@@ -3327,34 +3327,34 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C5" s="24" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="D5" s="23" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E5" s="24" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H5" s="23" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J5" s="23" t="n">
         <v>11</v>
       </c>
       <c r="K5" s="24" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -3364,28 +3364,28 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D6" s="23" t="n">
+        <v>42</v>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>49</v>
+      </c>
+      <c r="F6" s="23" t="n">
         <v>40</v>
       </c>
-      <c r="E6" s="24" t="n">
-        <v>48</v>
-      </c>
-      <c r="F6" s="23" t="n">
-        <v>38</v>
-      </c>
       <c r="G6" s="24" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H6" s="23" t="n">
         <v>18</v>
       </c>
       <c r="I6" s="24" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J6" s="23" t="n">
         <v>7</v>
@@ -3401,34 +3401,34 @@
         </is>
       </c>
       <c r="B7" s="23" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C7" s="24" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D7" s="23" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E7" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="G7" s="24" t="n">
         <v>48</v>
       </c>
-      <c r="F7" s="23" t="n">
-        <v>39</v>
-      </c>
-      <c r="G7" s="24" t="n">
-        <v>46</v>
-      </c>
       <c r="H7" s="23" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I7" s="24" t="n">
         <v>22</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K7" s="24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -3438,31 +3438,31 @@
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C8" s="24" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E8" s="24" t="n">
+        <v>57</v>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>46</v>
+      </c>
+      <c r="G8" s="24" t="n">
         <v>55</v>
       </c>
-      <c r="F8" s="23" t="n">
-        <v>44</v>
-      </c>
-      <c r="G8" s="24" t="n">
-        <v>53</v>
-      </c>
       <c r="H8" s="23" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J8" s="23" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K8" s="24" t="n">
         <v>9</v>
@@ -3475,13 +3475,13 @@
         </is>
       </c>
       <c r="B9" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="C9" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="C9" s="24" t="n">
-        <v>9</v>
-      </c>
       <c r="D9" s="23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E9" s="24" t="n">
         <v>11</v>
@@ -3502,7 +3502,7 @@
         <v>2</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -3512,34 +3512,34 @@
         </is>
       </c>
       <c r="B10" s="23" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C10" s="24" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D10" s="23" t="n">
+        <v>53</v>
+      </c>
+      <c r="E10" s="24" t="n">
+        <v>63</v>
+      </c>
+      <c r="F10" s="23" t="n">
         <v>51</v>
       </c>
-      <c r="E10" s="24" t="n">
-        <v>61</v>
-      </c>
-      <c r="F10" s="23" t="n">
-        <v>49</v>
-      </c>
       <c r="G10" s="24" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I10" s="24" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J10" s="23" t="n">
         <v>8</v>
       </c>
       <c r="K10" s="24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -3549,31 +3549,31 @@
         </is>
       </c>
       <c r="B11" s="23" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C11" s="24" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E11" s="24" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F11" s="23" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H11" s="23" t="n">
         <v>18</v>
       </c>
       <c r="I11" s="24" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J11" s="23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K11" s="24" t="n">
         <v>8</v>
@@ -3586,22 +3586,22 @@
         </is>
       </c>
       <c r="B12" s="23" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C12" s="24" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D12" s="23" t="n">
         <v>25</v>
       </c>
       <c r="E12" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" s="23" t="n">
+        <v>24</v>
+      </c>
+      <c r="G12" s="24" t="n">
         <v>29</v>
-      </c>
-      <c r="F12" s="23" t="n">
-        <v>23</v>
-      </c>
-      <c r="G12" s="24" t="n">
-        <v>28</v>
       </c>
       <c r="H12" s="23" t="n">
         <v>11</v>
@@ -3610,10 +3610,10 @@
         <v>13</v>
       </c>
       <c r="J12" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K12" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -3623,28 +3623,28 @@
         </is>
       </c>
       <c r="B13" s="23" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C13" s="24" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D13" s="23" t="n">
+        <v>44</v>
+      </c>
+      <c r="E13" s="24" t="n">
+        <v>52</v>
+      </c>
+      <c r="F13" s="23" t="n">
         <v>42</v>
       </c>
-      <c r="E13" s="24" t="n">
-        <v>50</v>
-      </c>
-      <c r="F13" s="23" t="n">
-        <v>40</v>
-      </c>
       <c r="G13" s="24" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H13" s="23" t="n">
         <v>19</v>
       </c>
       <c r="I13" s="24" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J13" s="23" t="n">
         <v>7</v>
@@ -3660,34 +3660,34 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>278</v>
+        <v>243</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>331</v>
+        <v>289</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>422</v>
+        <v>437</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>338</v>
+        <v>351</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>403</v>
+        <v>417</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16">
@@ -3726,7 +3726,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C18" t="n">
         <v>244</v>
@@ -3793,7 +3793,7 @@
         <v>31</v>
       </c>
       <c r="C22" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D22" t="n">
         <v>14</v>
@@ -3822,10 +3822,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C24" t="n">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D24" t="n">
         <v>60.4</v>
@@ -3857,7 +3857,7 @@
         <v>141</v>
       </c>
       <c r="C26" t="n">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D26" t="n">
         <v>64.09999999999999</v>
@@ -4041,10 +4041,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>973</v>
+        <v>962</v>
       </c>
       <c r="D14" t="n">
-        <v>1156</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="15">
@@ -4059,10 +4059,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>216</v>
+        <v>225</v>
       </c>
       <c r="D15" t="n">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="16">
@@ -4073,16 +4073,16 @@
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="D16" t="n">
-        <v>1413</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>── ASIGNACIÓN AL MÁXIMO (1413 und) ──</t>
+          <t>── ASIGNACIÓN AL MÁXIMO (1410 und) ──</t>
         </is>
       </c>
     </row>
@@ -4115,7 +4115,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>408</v>
+        <v>396</v>
       </c>
     </row>
     <row r="22">
@@ -4125,7 +4125,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="23">
@@ -4135,7 +4135,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>665</v>
+        <v>662</v>
       </c>
     </row>
     <row r="24">
@@ -4145,7 +4145,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1413</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="25">
@@ -4155,7 +4155,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="27">
@@ -4166,7 +4166,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>1189 – 1413 und</t>
+          <t>1187 – 1410 und</t>
         </is>
       </c>
     </row>
@@ -4430,7 +4430,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Al máximo (1413 und) quedan 79 cierres remanentes.</t>
+          <t xml:space="preserve">   Al máximo (1410 und) quedan 82 cierres remanentes.</t>
         </is>
       </c>
     </row>
@@ -4447,14 +4447,14 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Compromiso mín: 1189 und.</t>
+          <t xml:space="preserve">   Compromiso mín: 1187 und.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Techo máx: 1413 und.</t>
+          <t xml:space="preserve">   Techo máx: 1410 und.</t>
         </is>
       </c>
     </row>
@@ -4478,14 +4478,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">   XL reforzado +1.5 pp desde L → L 13.3% · XL 4.9%.</t>
+          <t xml:space="preserve">   XL reforzado +1.5 pp desde L → L 13.8% · XL 5.1%.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Núcleo S+M: +0.75 pp a S y a M (igual en chaqueta y pant); resto desde XS/L/XL proporcional.</t>
+          <t xml:space="preserve">   XS objetivo 20.5%: exceso de XS repartido por igual a S y M (criterio I+D).</t>
         </is>
       </c>
     </row>

</xml_diff>